<commit_message>
[cubicon] v1.5.0-rc5: fix dark-mode splash logo (remove legacy "style" wordmark)
- splash_logo_dark.png was the legacy "style CUBICON" logo; the Style series is a Cubicon
  legacy printer brand not supported by OrcaForCubicon. Replaced with a dark-mode CUBICON
  logo derived from the light logo (white CUBICON wordmark + colored icon, transparent
  background, 2495->2125px), so the dark splash no longer shows "style".
- Bump product version rc4 -> rc5; update Excel release notes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
+++ b/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc4</t>
+          <t>1.5.0-rc5</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -547,29 +547,29 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Build / Filament</t>
+          <t>Splash</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>테스트 전용 필라멘트 분리 (test 빌드=포함 / release 빌드=제외)</t>
+          <t>다크모드 스플래시 로고에서 legacy 'style' 문구 제거</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>cubicon/version/test_only_filaments.txt 매니페스트에 나열한 미검증 필라멘트를 release 빌드에서만 제거(cubicon/scripts/prune_test_filaments.ps1, build_win.ps1 -BuildType release 에서 호출). SSOT(cubicon/resources)는 전부 유지 → test 빌드는 모두 포함. 현재 test 전용: Cubicon Rainbow PLA HS, Cubicon TPU-HS(+fdm_filament_tpu). 검증 완료 시 매니페스트에서 해당 줄만 삭제하면 정식 승격.</t>
+          <t>splash_logo_dark.png 가 큐비콘 legacy 'style CUBICON' 로고였음(Style 시리즈는 OrcaForCubicon 미지원). light 로고 기반으로 흰색 CUBICON 텍스트 + 컬러 아이콘의 다크모드 전용 로고로 교체(2495→2125px).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc4</t>
+          <t>1.5.0-rc5</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -589,19 +589,19 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc3 → rc4</t>
+          <t>제품 버전 rc4 → rc5</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>테스트/정식 필라멘트 분리 기능 반영.</t>
+          <t>다크모드 스플래시 로고 수정 반영.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc3</t>
+          <t>1.5.0-rc4</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -616,24 +616,24 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Update check</t>
+          <t>Build / Filament</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>OrcaForCubicon 전용 업데이트 알림 기능 (OrcaSlicer 기본 체크 비활성화)</t>
+          <t>테스트 전용 필라멘트 분리 (test 빌드=포함 / release 빌드=제외)</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>실행 시 GitHub 최신 릴리스(api.github.com/repos/Hyvision/OrcaForCubicon/releases/latest)를 조회해 제품버전 CUBI_ORCA_VERSION 과 비교, 새 정식 릴리스가 있으면 팝업 알림 → '다운로드' 시 브라우저로 릴리스 페이지 열기. 정식 릴리스만 대상(/releases/latest 가 draft·prerelease 자동 제외). OrcaSlicer 의 check_new_version_sf 는 시작·수동 '업데이트 확인' 메뉴 양쪽에서 check_new_version_cubicon 으로 대체. 기존 UpdateVersionDialog 재사용. (patch 0009) ※ 동작하려면 레포 public 전환 + GitHub Releases 발행 필요.</t>
+          <t>cubicon/version/test_only_filaments.txt 매니페스트에 나열한 미검증 필라멘트를 release 빌드에서만 제거(cubicon/scripts/prune_test_filaments.ps1, build_win.ps1 -BuildType release 에서 호출). SSOT(cubicon/resources)는 전부 유지 → test 빌드는 모두 포함. 현재 test 전용: Cubicon Rainbow PLA HS, Cubicon TPU-HS(+fdm_filament_tpu). 검증 완료 시 매니페스트에서 해당 줄만 삭제하면 정식 승격.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc3</t>
+          <t>1.5.0-rc4</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -653,19 +653,19 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc2 → rc3</t>
+          <t>제품 버전 rc3 → rc4</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>업데이트 알림 기능 추가 반영.</t>
+          <t>테스트/정식 필라멘트 분리 기능 반영.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc2</t>
+          <t>1.5.0-rc3</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -675,29 +675,29 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>G-code / Mainsail</t>
+          <t>Update check</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>G-code 헤더 슬라이서명·버전 정정 (Moonraker 메타데이터 파싱 복원)</t>
+          <t>OrcaForCubicon 전용 업데이트 알림 기능 (OrcaSlicer 기본 체크 비활성화)</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>header_slic3r_generated() 가 "OrcaForCubicon 2.4.2" → "OrcaSlicer &lt;제품버전&gt;" 로 변경. Moonraker/Mainsail 은 인식된 슬라이서명(OrcaSlicer 등)일 때만 슬라이싱 정보를 파싱함 → 기존엔 Unknown+정보 없음. 버전도 Orca 2.4.2 대신 재정의 제품버전 표기. Orca 자체 재파싱은 GCodeProcessor 의 "generated by OrcaSlicer" producer 태그로 유지. (patch 0008)</t>
+          <t>실행 시 GitHub 최신 릴리스(api.github.com/repos/Hyvision/OrcaForCubicon/releases/latest)를 조회해 제품버전 CUBI_ORCA_VERSION 과 비교, 새 정식 릴리스가 있으면 팝업 알림 → '다운로드' 시 브라우저로 릴리스 페이지 열기. 정식 릴리스만 대상(/releases/latest 가 draft·prerelease 자동 제외). OrcaSlicer 의 check_new_version_sf 는 시작·수동 '업데이트 확인' 메뉴 양쪽에서 check_new_version_cubicon 으로 대체. 기존 UpdateVersionDialog 재사용. (patch 0009) ※ 동작하려면 레포 public 전환 + GitHub Releases 발행 필요.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc2</t>
+          <t>1.5.0-rc3</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -707,22 +707,22 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>build_win.ps1</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>release / test 빌드 유형 옵션 추가</t>
+          <t>제품 버전 rc2 → rc3</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>-BuildType test|release (대화식 프롬프트 4번). release 는 버전의 -rc 접미사를 제거하여 splash·버전정보·About 대화상자·G-code 헤더·인스톨러명 모두에 반영. test 는 rc 유지. cubicon_version.txt(SSOT)를 빌드 중 임시 수정 후 finally 에서 원복.</t>
+          <t>업데이트 알림 기능 추가 반영.</t>
         </is>
       </c>
     </row>
@@ -739,22 +739,22 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>build_win.ps1</t>
+          <t>G-code / Mainsail</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>병렬 컴파일 잡을 메모리 기준으로도 제한 (-MemPerJobGB)</t>
+          <t>G-code 헤더 슬라이서명·버전 정정 (Moonraker 메타데이터 파싱 복원)</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>28코어/32GB 환경에서 CpuPercent 70%(=19잡)로 libslic3r PCH 컴파일 시 페이지파일 고갈(C3859/C1076/OS 1455) 발생. jobs = min(CPU 상한, floor((총RAM-4)/MemPerJobGB[기본3])) 로 제한하여 재발 방지.</t>
+          <t>header_slic3r_generated() 가 "OrcaForCubicon 2.4.2" → "OrcaSlicer &lt;제품버전&gt;" 로 변경. Moonraker/Mainsail 은 인식된 슬라이서명(OrcaSlicer 등)일 때만 슬라이싱 정보를 파싱함 → 기존엔 Unknown+정보 없음. 버전도 Orca 2.4.2 대신 재정의 제품버전 표기. Orca 자체 재파싱은 GCodeProcessor 의 "generated by OrcaSlicer" producer 태그로 유지. (patch 0008)</t>
         </is>
       </c>
     </row>
@@ -771,29 +771,29 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>build_win.ps1</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc1 → rc2</t>
+          <t>release / test 빌드 유형 옵션 추가</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>cubicon/version/cubicon_version.txt. 규칙: 매 수정마다 rc 1 증가(반영 여부 식별용).</t>
+          <t>-BuildType test|release (대화식 프롬프트 4번). release 는 버전의 -rc 접미사를 제거하여 splash·버전정보·About 대화상자·G-code 헤더·인스톨러명 모두에 반영. test 는 rc 유지. cubicon_version.txt(SSOT)를 빌드 중 임시 수정 후 finally 에서 원복.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc1</t>
+          <t>1.5.0-rc2</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -803,29 +803,29 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Machine profile</t>
+          <t>build_win.ps1</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>장비 Max Jerk 하향 (Bambu·Creality 기조: 고가감속·저저크)</t>
+          <t>병렬 컴파일 잡을 메모리 기준으로도 제한 (-MemPerJobGB)</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>xCeler-Plus/I/Mini 3종: X 20→5, Y 20→5, Z 20→2, E 20→2.5 mm/s. 캔틸레버 베드 편심 틸트로 레이어 중 Z가 상시 반전할 때 높은 Z 저크가 임펄스 진동→수직 벽면 잔상(ghosting)을 유발하던 문제 해결. 장비 프로파일 version → 1.5.0.</t>
+          <t>28코어/32GB 환경에서 CpuPercent 70%(=19잡)로 libslic3r PCH 컴파일 시 페이지파일 고갈(C3859/C1076/OS 1455) 발생. jobs = min(CPU 상한, floor((총RAM-4)/MemPerJobGB[기본3])) 로 제한하여 재발 방지.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc1</t>
+          <t>1.5.0-rc2</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -835,22 +835,22 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Filament profile</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>신규 필라멘트: Cubicon TPU-HS</t>
+          <t>제품 버전 rc1 → rc2</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>isun3d TPU-HS(고속 TPU, Shore 95A) 추가. base + xCeler-I/Plus/Mini. fdm_filament_tpu 계열 베이스 신설. 초기값(노즐 230/230, 베드 50, 최대유량 5, 팬 100%) — 캘리브레이션 예정.</t>
+          <t>cubicon/version/cubicon_version.txt. 규칙: 매 수정마다 rc 1 증가(반영 여부 식별용).</t>
         </is>
       </c>
     </row>
@@ -872,17 +872,17 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Filament profile</t>
+          <t>Machine profile</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>신규 필라멘트: Cubicon Rainbow PLA HS</t>
+          <t>장비 Max Jerk 하향 (Bambu·Creality 기조: 고가감속·저저크)</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>한일 Rainbow PLA High Speed (Bambu PLA HS 유사). base + xCeler-I/Plus/Mini, Cubicon PLA @base 상속. 초기값(노즐 220/215, 베드 60, 최대유량 28, flow 0.98) — 캘리브레이션 예정.</t>
+          <t>xCeler-Plus/I/Mini 3종: X 20→5, Y 20→5, Z 20→2, E 20→2.5 mm/s. 캔틸레버 베드 편심 틸트로 레이어 중 Z가 상시 반전할 때 높은 Z 저크가 임펄스 진동→수직 벽면 잔상(ghosting)을 유발하던 문제 해결. 장비 프로파일 version → 1.5.0.</t>
         </is>
       </c>
     </row>
@@ -899,20 +899,84 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
+          <t>Feat</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Filament profile</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>신규 필라멘트: Cubicon TPU-HS</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>isun3d TPU-HS(고속 TPU, Shore 95A) 추가. base + xCeler-I/Plus/Mini. fdm_filament_tpu 계열 베이스 신설. 초기값(노즐 230/230, 베드 50, 최대유량 5, 팬 100%) — 캘리브레이션 예정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>1.5.0-rc1</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Feat</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Filament profile</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>신규 필라멘트: Cubicon Rainbow PLA HS</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>한일 Rainbow PLA High Speed (Bambu PLA HS 유사). base + xCeler-I/Plus/Mini, Cubicon PLA @base 상속. 초기값(노즐 220/215, 베드 60, 최대유량 28, flow 0.98) — 캘리브레이션 예정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>1.5.0-rc1</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
           <t>Chore</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>Profile package</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>프로파일 패키지 버전 02.03.02.00 → 02.03.03.00</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>Cubicon.json. 기설치 사용자에게 프로파일 갱신 전파를 위해 패키지 버전 상승 (신규 필라멘트·저크 반영).</t>
         </is>

</xml_diff>

<commit_message>
[cubicon] v1.5.1-rc1: bump base version to 1.5.1
Start of the 1.5.1 dev cycle. Published alongside v1.5.0 on GitHub Releases to verify
the OrcaForCubicon update-notification end-to-end: running v1.5.0 should detect v1.5.1
as newer and show the update popup.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
+++ b/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc5</t>
+          <t>1.5.1-rc1</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -547,22 +547,22 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Splash</t>
+          <t>version / release</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>다크모드 스플래시 로고에서 legacy 'style' 문구 제거</t>
+          <t>기본 버전 1.5.0 → 1.5.1 (다음 개발 사이클 시작)</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>splash_logo_dark.png 가 큐비콘 legacy 'style CUBICON' 로고였음(Style 시리즈는 OrcaForCubicon 미지원). light 로고 기반으로 흰색 CUBICON 텍스트 + 컬러 아이콘의 다크모드 전용 로고로 교체(2495→2125px).</t>
+          <t>GitHub v1.5.0 발행 후 v1.5.1 을 추가 발행하여, v1.5.0 실행 시 업데이트 알림 팝업이 정상 동작하는지 end-to-end 검증하기 위한 버전 업. release 빌드 시 '1.5.1' 로 태깅.</t>
         </is>
       </c>
     </row>
@@ -579,29 +579,29 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>Splash</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc4 → rc5</t>
+          <t>다크모드 스플래시 로고에서 legacy 'style' 문구 제거</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>다크모드 스플래시 로고 수정 반영.</t>
+          <t>splash_logo_dark.png 가 큐비콘 legacy 'style CUBICON' 로고였음(Style 시리즈는 OrcaForCubicon 미지원). light 로고 기반으로 흰색 CUBICON 텍스트 + 컬러 아이콘의 다크모드 전용 로고로 교체(2495→2125px).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc4</t>
+          <t>1.5.0-rc5</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -611,22 +611,22 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Build / Filament</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>테스트 전용 필라멘트 분리 (test 빌드=포함 / release 빌드=제외)</t>
+          <t>제품 버전 rc4 → rc5</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>cubicon/version/test_only_filaments.txt 매니페스트에 나열한 미검증 필라멘트를 release 빌드에서만 제거(cubicon/scripts/prune_test_filaments.ps1, build_win.ps1 -BuildType release 에서 호출). SSOT(cubicon/resources)는 전부 유지 → test 빌드는 모두 포함. 현재 test 전용: Cubicon Rainbow PLA HS, Cubicon TPU-HS(+fdm_filament_tpu). 검증 완료 시 매니페스트에서 해당 줄만 삭제하면 정식 승격.</t>
+          <t>다크모드 스플래시 로고 수정 반영.</t>
         </is>
       </c>
     </row>
@@ -643,29 +643,29 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>Build / Filament</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc3 → rc4</t>
+          <t>테스트 전용 필라멘트 분리 (test 빌드=포함 / release 빌드=제외)</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>테스트/정식 필라멘트 분리 기능 반영.</t>
+          <t>cubicon/version/test_only_filaments.txt 매니페스트에 나열한 미검증 필라멘트를 release 빌드에서만 제거(cubicon/scripts/prune_test_filaments.ps1, build_win.ps1 -BuildType release 에서 호출). SSOT(cubicon/resources)는 전부 유지 → test 빌드는 모두 포함. 현재 test 전용: Cubicon Rainbow PLA HS, Cubicon TPU-HS(+fdm_filament_tpu). 검증 완료 시 매니페스트에서 해당 줄만 삭제하면 정식 승격.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc3</t>
+          <t>1.5.0-rc4</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -675,22 +675,22 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Update check</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>OrcaForCubicon 전용 업데이트 알림 기능 (OrcaSlicer 기본 체크 비활성화)</t>
+          <t>제품 버전 rc3 → rc4</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>실행 시 GitHub 최신 릴리스(api.github.com/repos/Hyvision/OrcaForCubicon/releases/latest)를 조회해 제품버전 CUBI_ORCA_VERSION 과 비교, 새 정식 릴리스가 있으면 팝업 알림 → '다운로드' 시 브라우저로 릴리스 페이지 열기. 정식 릴리스만 대상(/releases/latest 가 draft·prerelease 자동 제외). OrcaSlicer 의 check_new_version_sf 는 시작·수동 '업데이트 확인' 메뉴 양쪽에서 check_new_version_cubicon 으로 대체. 기존 UpdateVersionDialog 재사용. (patch 0009) ※ 동작하려면 레포 public 전환 + GitHub Releases 발행 필요.</t>
+          <t>테스트/정식 필라멘트 분리 기능 반영.</t>
         </is>
       </c>
     </row>
@@ -707,29 +707,29 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>Update check</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc2 → rc3</t>
+          <t>OrcaForCubicon 전용 업데이트 알림 기능 (OrcaSlicer 기본 체크 비활성화)</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>업데이트 알림 기능 추가 반영.</t>
+          <t>실행 시 GitHub 최신 릴리스(api.github.com/repos/Hyvision/OrcaForCubicon/releases/latest)를 조회해 제품버전 CUBI_ORCA_VERSION 과 비교, 새 정식 릴리스가 있으면 팝업 알림 → '다운로드' 시 브라우저로 릴리스 페이지 열기. 정식 릴리스만 대상(/releases/latest 가 draft·prerelease 자동 제외). OrcaSlicer 의 check_new_version_sf 는 시작·수동 '업데이트 확인' 메뉴 양쪽에서 check_new_version_cubicon 으로 대체. 기존 UpdateVersionDialog 재사용. (patch 0009) ※ 동작하려면 레포 public 전환 + GitHub Releases 발행 필요.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc2</t>
+          <t>1.5.0-rc3</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -739,22 +739,22 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>G-code / Mainsail</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>G-code 헤더 슬라이서명·버전 정정 (Moonraker 메타데이터 파싱 복원)</t>
+          <t>제품 버전 rc2 → rc3</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>header_slic3r_generated() 가 "OrcaForCubicon 2.4.2" → "OrcaSlicer &lt;제품버전&gt;" 로 변경. Moonraker/Mainsail 은 인식된 슬라이서명(OrcaSlicer 등)일 때만 슬라이싱 정보를 파싱함 → 기존엔 Unknown+정보 없음. 버전도 Orca 2.4.2 대신 재정의 제품버전 표기. Orca 자체 재파싱은 GCodeProcessor 의 "generated by OrcaSlicer" producer 태그로 유지. (patch 0008)</t>
+          <t>업데이트 알림 기능 추가 반영.</t>
         </is>
       </c>
     </row>
@@ -771,22 +771,22 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>build_win.ps1</t>
+          <t>G-code / Mainsail</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>release / test 빌드 유형 옵션 추가</t>
+          <t>G-code 헤더 슬라이서명·버전 정정 (Moonraker 메타데이터 파싱 복원)</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>-BuildType test|release (대화식 프롬프트 4번). release 는 버전의 -rc 접미사를 제거하여 splash·버전정보·About 대화상자·G-code 헤더·인스톨러명 모두에 반영. test 는 rc 유지. cubicon_version.txt(SSOT)를 빌드 중 임시 수정 후 finally 에서 원복.</t>
+          <t>header_slic3r_generated() 가 "OrcaForCubicon 2.4.2" → "OrcaSlicer &lt;제품버전&gt;" 로 변경. Moonraker/Mainsail 은 인식된 슬라이서명(OrcaSlicer 등)일 때만 슬라이싱 정보를 파싱함 → 기존엔 Unknown+정보 없음. 버전도 Orca 2.4.2 대신 재정의 제품버전 표기. Orca 자체 재파싱은 GCodeProcessor 의 "generated by OrcaSlicer" producer 태그로 유지. (patch 0008)</t>
         </is>
       </c>
     </row>
@@ -813,12 +813,12 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>병렬 컴파일 잡을 메모리 기준으로도 제한 (-MemPerJobGB)</t>
+          <t>release / test 빌드 유형 옵션 추가</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>28코어/32GB 환경에서 CpuPercent 70%(=19잡)로 libslic3r PCH 컴파일 시 페이지파일 고갈(C3859/C1076/OS 1455) 발생. jobs = min(CPU 상한, floor((총RAM-4)/MemPerJobGB[기본3])) 로 제한하여 재발 방지.</t>
+          <t>-BuildType test|release (대화식 프롬프트 4번). release 는 버전의 -rc 접미사를 제거하여 splash·버전정보·About 대화상자·G-code 헤더·인스톨러명 모두에 반영. test 는 rc 유지. cubicon_version.txt(SSOT)를 빌드 중 임시 수정 후 finally 에서 원복.</t>
         </is>
       </c>
     </row>
@@ -835,29 +835,29 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>build_win.ps1</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc1 → rc2</t>
+          <t>병렬 컴파일 잡을 메모리 기준으로도 제한 (-MemPerJobGB)</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>cubicon/version/cubicon_version.txt. 규칙: 매 수정마다 rc 1 증가(반영 여부 식별용).</t>
+          <t>28코어/32GB 환경에서 CpuPercent 70%(=19잡)로 libslic3r PCH 컴파일 시 페이지파일 고갈(C3859/C1076/OS 1455) 발생. jobs = min(CPU 상한, floor((총RAM-4)/MemPerJobGB[기본3])) 로 제한하여 재발 방지.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc1</t>
+          <t>1.5.0-rc2</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -867,22 +867,22 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Machine profile</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>장비 Max Jerk 하향 (Bambu·Creality 기조: 고가감속·저저크)</t>
+          <t>제품 버전 rc1 → rc2</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>xCeler-Plus/I/Mini 3종: X 20→5, Y 20→5, Z 20→2, E 20→2.5 mm/s. 캔틸레버 베드 편심 틸트로 레이어 중 Z가 상시 반전할 때 높은 Z 저크가 임펄스 진동→수직 벽면 잔상(ghosting)을 유발하던 문제 해결. 장비 프로파일 version → 1.5.0.</t>
+          <t>cubicon/version/cubicon_version.txt. 규칙: 매 수정마다 rc 1 증가(반영 여부 식별용).</t>
         </is>
       </c>
     </row>
@@ -904,17 +904,17 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Filament profile</t>
+          <t>Machine profile</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>신규 필라멘트: Cubicon TPU-HS</t>
+          <t>장비 Max Jerk 하향 (Bambu·Creality 기조: 고가감속·저저크)</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>isun3d TPU-HS(고속 TPU, Shore 95A) 추가. base + xCeler-I/Plus/Mini. fdm_filament_tpu 계열 베이스 신설. 초기값(노즐 230/230, 베드 50, 최대유량 5, 팬 100%) — 캘리브레이션 예정.</t>
+          <t>xCeler-Plus/I/Mini 3종: X 20→5, Y 20→5, Z 20→2, E 20→2.5 mm/s. 캔틸레버 베드 편심 틸트로 레이어 중 Z가 상시 반전할 때 높은 Z 저크가 임펄스 진동→수직 벽면 잔상(ghosting)을 유발하던 문제 해결. 장비 프로파일 version → 1.5.0.</t>
         </is>
       </c>
     </row>
@@ -941,12 +941,12 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>신규 필라멘트: Cubicon Rainbow PLA HS</t>
+          <t>신규 필라멘트: Cubicon TPU-HS</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>한일 Rainbow PLA High Speed (Bambu PLA HS 유사). base + xCeler-I/Plus/Mini, Cubicon PLA @base 상속. 초기값(노즐 220/215, 베드 60, 최대유량 28, flow 0.98) — 캘리브레이션 예정.</t>
+          <t>isun3d TPU-HS(고속 TPU, Shore 95A) 추가. base + xCeler-I/Plus/Mini. fdm_filament_tpu 계열 베이스 신설. 초기값(노즐 230/230, 베드 50, 최대유량 5, 팬 100%) — 캘리브레이션 예정.</t>
         </is>
       </c>
     </row>
@@ -963,20 +963,52 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
+          <t>Feat</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Filament profile</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>신규 필라멘트: Cubicon Rainbow PLA HS</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>한일 Rainbow PLA High Speed (Bambu PLA HS 유사). base + xCeler-I/Plus/Mini, Cubicon PLA @base 상속. 초기값(노즐 220/215, 베드 60, 최대유량 28, flow 0.98) — 캘리브레이션 예정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>1.5.0-rc1</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
           <t>Chore</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>Profile package</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>프로파일 패키지 버전 02.03.02.00 → 02.03.03.00</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>Cubicon.json. 기설치 사용자에게 프로파일 갱신 전파를 위해 패키지 버전 상승 (신규 필라멘트·저크 반영).</t>
         </is>

</xml_diff>

<commit_message>
[cubicon] v1.5.1-rc3: apply Rainbow PLA HS calibration to the profile
Cubicon Rainbow PLA HS @base updated with the calibration-confirmed values:
- filament_max_volumetric_speed 28 -> 17 mm3/s (measured max-flow test)
- enable_pressure_advance + pressure_advance 0.03 (new; PA pattern ~0.035 -> 0.03)
- nozzle 215/220, bed 60, flow 0.98 already matched; retraction 2mm inherited from PLA base.
Still test-only (excluded from release builds until verified). Detailed report:
cubicon/profile/Rainbow PLA HS_ProfileUpdate_20260731_R0.pptx.

Bump product version rc2 -> rc3; update Excel release notes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
+++ b/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,64 +537,64 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1.5.1-rc2</t>
+          <t>1.5.1-rc3</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>G-code load</t>
+          <t>Filament profile</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>OrcaForCubicon(1.4.1 등) 및 신규 1.5.0 gcode 로드 실패 수정 (patch 0008 회귀 대응)</t>
+          <t>Rainbow PLA HS 캘리브레이션 확정값 반영</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>patch 0008 로 헤더를 '; generated by OrcaSlicer'로 바꾼 뒤, Config.cpp 의 로드 검증이 여전히 '; generated by OrcaForCubicon' 만 허용해 자기 파일조차 'Not a gcode file generated by OrcaForCubicon' 로 거부되던 문제. 검증에 '; generated by ' + SLIC3R_OFFICIAL_NAME('OrcaSlicer') 허용을 추가(patch 0008 갱신).</t>
+          <t>Cubicon Rainbow PLA HS @base: 최대 체적 속도 28→17 mm³/s(실측), Pressure Advance 0.03 신규 활성화. 온도(215/220)·베드(60)·유량비율(0.98)·후퇴(2mm 상속)는 캘리브레이션으로 적정 확인. 여전히 test-only. 상세: Rainbow PLA HS_ProfileUpdate_20260731_R0.pptx.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc2</t>
+          <t>1.5.1-rc3</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Installer / Runtime</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>WebView2 Evergreen 런타임 조건부 설치 추가 (마법사 blank 방지)</t>
+          <t>제품 버전 rc2 → rc3</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>WebView2Loader.dll 만으로는 부족 — 클린 PC에 WebView2 런타임이 없으면 설정 마법사가 blank. NSIS 에서 레지스트리(EdgeUpdate pv) 확인 후 미설치 시 MicrosoftEdgeWebview2Setup.exe 를 silent 설치. package_win.ps1 이 부트스트래퍼를 자동 다운로드해 번들. (VC++ CRT/.NET-런타임 이슈는 CopyRuntime+vc_redist 로 기존에 이미 처리됨)</t>
+          <t>Rainbow PLA HS 프로파일 캘리브레이션 반영.</t>
         </is>
       </c>
     </row>
@@ -611,29 +611,29 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>G-code load</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>제품 버전 rc1 → rc2</t>
+          <t>OrcaForCubicon(1.4.1 등) 및 신규 1.5.0 gcode 로드 실패 수정 (patch 0008 회귀 대응)</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>gcode 로드 수정 + WebView2 런타임 준비 반영.</t>
+          <t>patch 0008 로 헤더를 '; generated by OrcaSlicer'로 바꾼 뒤, Config.cpp 의 로드 검증이 여전히 '; generated by OrcaForCubicon' 만 허용해 자기 파일조차 'Not a gcode file generated by OrcaForCubicon' 로 거부되던 문제. 검증에 '; generated by ' + SLIC3R_OFFICIAL_NAME('OrcaSlicer') 허용을 추가(patch 0008 갱신).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc1</t>
+          <t>1.5.1-rc2</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -643,29 +643,29 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>version / release</t>
+          <t>Installer / Runtime</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>기본 버전 1.5.0 → 1.5.1 (다음 개발 사이클 시작)</t>
+          <t>WebView2 Evergreen 런타임 조건부 설치 추가 (마법사 blank 방지)</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>GitHub v1.5.0 발행 후 v1.5.1 을 추가 발행하여, v1.5.0 실행 시 업데이트 알림 팝업이 정상 동작하는지 end-to-end 검증하기 위한 버전 업. release 빌드 시 '1.5.1' 로 태깅.</t>
+          <t>WebView2Loader.dll 만으로는 부족 — 클린 PC에 WebView2 런타임이 없으면 설정 마법사가 blank. NSIS 에서 레지스트리(EdgeUpdate pv) 확인 후 미설치 시 MicrosoftEdgeWebview2Setup.exe 를 silent 설치. package_win.ps1 이 부트스트래퍼를 자동 다운로드해 번들. (VC++ CRT/.NET-런타임 이슈는 CopyRuntime+vc_redist 로 기존에 이미 처리됨)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc5</t>
+          <t>1.5.1-rc2</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -675,29 +675,29 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Splash</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>다크모드 스플래시 로고에서 legacy 'style' 문구 제거</t>
+          <t>제품 버전 rc1 → rc2</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>splash_logo_dark.png 가 큐비콘 legacy 'style CUBICON' 로고였음(Style 시리즈는 OrcaForCubicon 미지원). light 로고 기반으로 흰색 CUBICON 텍스트 + 컬러 아이콘의 다크모드 전용 로고로 교체(2495→2125px).</t>
+          <t>gcode 로드 수정 + WebView2 런타임 준비 반영.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc5</t>
+          <t>1.5.1-rc1</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -712,24 +712,24 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>version / release</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc4 → rc5</t>
+          <t>기본 버전 1.5.0 → 1.5.1 (다음 개발 사이클 시작)</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>다크모드 스플래시 로고 수정 반영.</t>
+          <t>GitHub v1.5.0 발행 후 v1.5.1 을 추가 발행하여, v1.5.0 실행 시 업데이트 알림 팝업이 정상 동작하는지 end-to-end 검증하기 위한 버전 업. release 빌드 시 '1.5.1' 로 태깅.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc4</t>
+          <t>1.5.0-rc5</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -739,29 +739,29 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Build / Filament</t>
+          <t>Splash</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>테스트 전용 필라멘트 분리 (test 빌드=포함 / release 빌드=제외)</t>
+          <t>다크모드 스플래시 로고에서 legacy 'style' 문구 제거</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>cubicon/version/test_only_filaments.txt 매니페스트에 나열한 미검증 필라멘트를 release 빌드에서만 제거(cubicon/scripts/prune_test_filaments.ps1, build_win.ps1 -BuildType release 에서 호출). SSOT(cubicon/resources)는 전부 유지 → test 빌드는 모두 포함. 현재 test 전용: Cubicon Rainbow PLA HS, Cubicon TPU-HS(+fdm_filament_tpu). 검증 완료 시 매니페스트에서 해당 줄만 삭제하면 정식 승격.</t>
+          <t>splash_logo_dark.png 가 큐비콘 legacy 'style CUBICON' 로고였음(Style 시리즈는 OrcaForCubicon 미지원). light 로고 기반으로 흰색 CUBICON 텍스트 + 컬러 아이콘의 다크모드 전용 로고로 교체(2495→2125px).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc4</t>
+          <t>1.5.0-rc5</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -781,19 +781,19 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc3 → rc4</t>
+          <t>제품 버전 rc4 → rc5</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>테스트/정식 필라멘트 분리 기능 반영.</t>
+          <t>다크모드 스플래시 로고 수정 반영.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc3</t>
+          <t>1.5.0-rc4</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -808,24 +808,24 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Update check</t>
+          <t>Build / Filament</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>OrcaForCubicon 전용 업데이트 알림 기능 (OrcaSlicer 기본 체크 비활성화)</t>
+          <t>테스트 전용 필라멘트 분리 (test 빌드=포함 / release 빌드=제외)</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>실행 시 GitHub 최신 릴리스(api.github.com/repos/Hyvision/OrcaForCubicon/releases/latest)를 조회해 제품버전 CUBI_ORCA_VERSION 과 비교, 새 정식 릴리스가 있으면 팝업 알림 → '다운로드' 시 브라우저로 릴리스 페이지 열기. 정식 릴리스만 대상(/releases/latest 가 draft·prerelease 자동 제외). OrcaSlicer 의 check_new_version_sf 는 시작·수동 '업데이트 확인' 메뉴 양쪽에서 check_new_version_cubicon 으로 대체. 기존 UpdateVersionDialog 재사용. (patch 0009) ※ 동작하려면 레포 public 전환 + GitHub Releases 발행 필요.</t>
+          <t>cubicon/version/test_only_filaments.txt 매니페스트에 나열한 미검증 필라멘트를 release 빌드에서만 제거(cubicon/scripts/prune_test_filaments.ps1, build_win.ps1 -BuildType release 에서 호출). SSOT(cubicon/resources)는 전부 유지 → test 빌드는 모두 포함. 현재 test 전용: Cubicon Rainbow PLA HS, Cubicon TPU-HS(+fdm_filament_tpu). 검증 완료 시 매니페스트에서 해당 줄만 삭제하면 정식 승격.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc3</t>
+          <t>1.5.0-rc4</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -845,19 +845,19 @@
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc2 → rc3</t>
+          <t>제품 버전 rc3 → rc4</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>업데이트 알림 기능 추가 반영.</t>
+          <t>테스트/정식 필라멘트 분리 기능 반영.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc2</t>
+          <t>1.5.0-rc3</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -867,29 +867,29 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>G-code / Mainsail</t>
+          <t>Update check</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>G-code 헤더 슬라이서명·버전 정정 (Moonraker 메타데이터 파싱 복원)</t>
+          <t>OrcaForCubicon 전용 업데이트 알림 기능 (OrcaSlicer 기본 체크 비활성화)</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>header_slic3r_generated() 가 "OrcaForCubicon 2.4.2" → "OrcaSlicer &lt;제품버전&gt;" 로 변경. Moonraker/Mainsail 은 인식된 슬라이서명(OrcaSlicer 등)일 때만 슬라이싱 정보를 파싱함 → 기존엔 Unknown+정보 없음. 버전도 Orca 2.4.2 대신 재정의 제품버전 표기. Orca 자체 재파싱은 GCodeProcessor 의 "generated by OrcaSlicer" producer 태그로 유지. (patch 0008)</t>
+          <t>실행 시 GitHub 최신 릴리스(api.github.com/repos/Hyvision/OrcaForCubicon/releases/latest)를 조회해 제품버전 CUBI_ORCA_VERSION 과 비교, 새 정식 릴리스가 있으면 팝업 알림 → '다운로드' 시 브라우저로 릴리스 페이지 열기. 정식 릴리스만 대상(/releases/latest 가 draft·prerelease 자동 제외). OrcaSlicer 의 check_new_version_sf 는 시작·수동 '업데이트 확인' 메뉴 양쪽에서 check_new_version_cubicon 으로 대체. 기존 UpdateVersionDialog 재사용. (patch 0009) ※ 동작하려면 레포 public 전환 + GitHub Releases 발행 필요.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc2</t>
+          <t>1.5.0-rc3</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -899,22 +899,22 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>build_win.ps1</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>release / test 빌드 유형 옵션 추가</t>
+          <t>제품 버전 rc2 → rc3</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>-BuildType test|release (대화식 프롬프트 4번). release 는 버전의 -rc 접미사를 제거하여 splash·버전정보·About 대화상자·G-code 헤더·인스톨러명 모두에 반영. test 는 rc 유지. cubicon_version.txt(SSOT)를 빌드 중 임시 수정 후 finally 에서 원복.</t>
+          <t>업데이트 알림 기능 추가 반영.</t>
         </is>
       </c>
     </row>
@@ -931,22 +931,22 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>build_win.ps1</t>
+          <t>G-code / Mainsail</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>병렬 컴파일 잡을 메모리 기준으로도 제한 (-MemPerJobGB)</t>
+          <t>G-code 헤더 슬라이서명·버전 정정 (Moonraker 메타데이터 파싱 복원)</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>28코어/32GB 환경에서 CpuPercent 70%(=19잡)로 libslic3r PCH 컴파일 시 페이지파일 고갈(C3859/C1076/OS 1455) 발생. jobs = min(CPU 상한, floor((총RAM-4)/MemPerJobGB[기본3])) 로 제한하여 재발 방지.</t>
+          <t>header_slic3r_generated() 가 "OrcaForCubicon 2.4.2" → "OrcaSlicer &lt;제품버전&gt;" 로 변경. Moonraker/Mainsail 은 인식된 슬라이서명(OrcaSlicer 등)일 때만 슬라이싱 정보를 파싱함 → 기존엔 Unknown+정보 없음. 버전도 Orca 2.4.2 대신 재정의 제품버전 표기. Orca 자체 재파싱은 GCodeProcessor 의 "generated by OrcaSlicer" producer 태그로 유지. (patch 0008)</t>
         </is>
       </c>
     </row>
@@ -963,29 +963,29 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>build_win.ps1</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc1 → rc2</t>
+          <t>release / test 빌드 유형 옵션 추가</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>cubicon/version/cubicon_version.txt. 규칙: 매 수정마다 rc 1 증가(반영 여부 식별용).</t>
+          <t>-BuildType test|release (대화식 프롬프트 4번). release 는 버전의 -rc 접미사를 제거하여 splash·버전정보·About 대화상자·G-code 헤더·인스톨러명 모두에 반영. test 는 rc 유지. cubicon_version.txt(SSOT)를 빌드 중 임시 수정 후 finally 에서 원복.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc1</t>
+          <t>1.5.0-rc2</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -995,29 +995,29 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Machine profile</t>
+          <t>build_win.ps1</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>장비 Max Jerk 하향 (Bambu·Creality 기조: 고가감속·저저크)</t>
+          <t>병렬 컴파일 잡을 메모리 기준으로도 제한 (-MemPerJobGB)</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>xCeler-Plus/I/Mini 3종: X 20→5, Y 20→5, Z 20→2, E 20→2.5 mm/s. 캔틸레버 베드 편심 틸트로 레이어 중 Z가 상시 반전할 때 높은 Z 저크가 임펄스 진동→수직 벽면 잔상(ghosting)을 유발하던 문제 해결. 장비 프로파일 version → 1.5.0.</t>
+          <t>28코어/32GB 환경에서 CpuPercent 70%(=19잡)로 libslic3r PCH 컴파일 시 페이지파일 고갈(C3859/C1076/OS 1455) 발생. jobs = min(CPU 상한, floor((총RAM-4)/MemPerJobGB[기본3])) 로 제한하여 재발 방지.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc1</t>
+          <t>1.5.0-rc2</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -1027,22 +1027,22 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Filament profile</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>신규 필라멘트: Cubicon TPU-HS</t>
+          <t>제품 버전 rc1 → rc2</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>isun3d TPU-HS(고속 TPU, Shore 95A) 추가. base + xCeler-I/Plus/Mini. fdm_filament_tpu 계열 베이스 신설. 초기값(노즐 230/230, 베드 50, 최대유량 5, 팬 100%) — 캘리브레이션 예정.</t>
+          <t>cubicon/version/cubicon_version.txt. 규칙: 매 수정마다 rc 1 증가(반영 여부 식별용).</t>
         </is>
       </c>
     </row>
@@ -1064,17 +1064,17 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Filament profile</t>
+          <t>Machine profile</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>신규 필라멘트: Cubicon Rainbow PLA HS</t>
+          <t>장비 Max Jerk 하향 (Bambu·Creality 기조: 고가감속·저저크)</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>한일 Rainbow PLA High Speed (Bambu PLA HS 유사). base + xCeler-I/Plus/Mini, Cubicon PLA @base 상속. 초기값(노즐 220/215, 베드 60, 최대유량 28, flow 0.98) — 캘리브레이션 예정.</t>
+          <t>xCeler-Plus/I/Mini 3종: X 20→5, Y 20→5, Z 20→2, E 20→2.5 mm/s. 캔틸레버 베드 편심 틸트로 레이어 중 Z가 상시 반전할 때 높은 Z 저크가 임펄스 진동→수직 벽면 잔상(ghosting)을 유발하던 문제 해결. 장비 프로파일 version → 1.5.0.</t>
         </is>
       </c>
     </row>
@@ -1091,20 +1091,84 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
+          <t>Feat</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Filament profile</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>신규 필라멘트: Cubicon TPU-HS</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>isun3d TPU-HS(고속 TPU, Shore 95A) 추가. base + xCeler-I/Plus/Mini. fdm_filament_tpu 계열 베이스 신설. 초기값(노즐 230/230, 베드 50, 최대유량 5, 팬 100%) — 캘리브레이션 예정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>1.5.0-rc1</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Feat</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Filament profile</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>신규 필라멘트: Cubicon Rainbow PLA HS</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>한일 Rainbow PLA High Speed (Bambu PLA HS 유사). base + xCeler-I/Plus/Mini, Cubicon PLA @base 상속. 초기값(노즐 220/215, 베드 60, 최대유량 28, flow 0.98) — 캘리브레이션 예정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>1.5.0-rc1</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
           <t>Chore</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>Profile package</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
         <is>
           <t>프로파일 패키지 버전 02.03.02.00 → 02.03.03.00</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="F24" s="7" t="inlineStr">
         <is>
           <t>Cubicon.json. 기설치 사용자에게 프로파일 갱신 전파를 위해 패키지 버전 상승 (신규 필라멘트·저크 반영).</t>
         </is>

</xml_diff>

<commit_message>
[cubicon] v1.5.1-rc4: apply precision/tolerance calibration to the base process
cubicon common @base (shared by all Cubicon processes, so this applies to every material):
- elefant_foot_compensation 0.15 -> 0.2
- elefant_foot_compensation_layers -> 2 (was inherited 1)
- xy_hole_compensation -> 0.2, xy_contour_compensation -> 0.02 (were 0)
resolution 0.012, slice_closing_radius 0.049, elefant_foot_layers_density 100%,
precise_outer_wall / precise_z_height on, arc-fitting off already matched (Image #4).
From the Rainbow PLA HS tolerance calibration; precision settings are process-scoped
(not per-filament), so they are shared across all materials by design.

Bump product version rc3 -> rc4; update Excel release notes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
+++ b/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1.5.1-rc3</t>
+          <t>1.5.1-rc4</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -552,24 +552,24 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Filament profile</t>
+          <t>Process profile</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Rainbow PLA HS 캘리브레이션 확정값 반영</t>
+          <t>정밀도(공차) 보정 기본 프로세스 반영 (전 재료 공통)</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Cubicon Rainbow PLA HS @base: 최대 체적 속도 28→17 mm³/s(실측), Pressure Advance 0.03 신규 활성화. 온도(215/220)·베드(60)·유량비율(0.98)·후퇴(2mm 상속)는 캘리브레이션으로 적정 확인. 여전히 test-only. 상세: Rainbow PLA HS_ProfileUpdate_20260731_R0.pptx.</t>
+          <t>cubicon common @base: 코끼리발 보정 0.15→0.2 · 보정 레이어 2 · X-Y 구멍 보정 0.2 · X-Y 윤곽 보상 0.02 추가. resolution 0.012 · slice_closing 0.049 · EF density 100% · 정밀한 벽/정확한 Z · 원호맞춤 off 는 기존 일치. Rainbow PLA HS 공차 캘리브레이션 결과이며 공정 설정이라 전 재료에 공통 적용됨.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc3</t>
+          <t>1.5.1-rc4</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -589,76 +589,76 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc2 → rc3</t>
+          <t>제품 버전 rc3 → rc4</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Rainbow PLA HS 프로파일 캘리브레이션 반영.</t>
+          <t>정밀도 공차 프로세스 반영.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>1.5.1-rc2</t>
+          <t>1.5.1-rc3</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>G-code load</t>
+          <t>Filament profile</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>OrcaForCubicon(1.4.1 등) 및 신규 1.5.0 gcode 로드 실패 수정 (patch 0008 회귀 대응)</t>
+          <t>Rainbow PLA HS 캘리브레이션 확정값 반영</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>patch 0008 로 헤더를 '; generated by OrcaSlicer'로 바꾼 뒤, Config.cpp 의 로드 검증이 여전히 '; generated by OrcaForCubicon' 만 허용해 자기 파일조차 'Not a gcode file generated by OrcaForCubicon' 로 거부되던 문제. 검증에 '; generated by ' + SLIC3R_OFFICIAL_NAME('OrcaSlicer') 허용을 추가(patch 0008 갱신).</t>
+          <t>Cubicon Rainbow PLA HS @base: 최대 체적 속도 28→17 mm³/s(실측), Pressure Advance 0.03 신규 활성화. 온도(215/220)·베드(60)·유량비율(0.98)·후퇴(2mm 상속)는 캘리브레이션으로 적정 확인. 여전히 test-only. 상세: Rainbow PLA HS_ProfileUpdate_20260731_R0.pptx.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc2</t>
+          <t>1.5.1-rc3</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Installer / Runtime</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>WebView2 Evergreen 런타임 조건부 설치 추가 (마법사 blank 방지)</t>
+          <t>제품 버전 rc2 → rc3</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>WebView2Loader.dll 만으로는 부족 — 클린 PC에 WebView2 런타임이 없으면 설정 마법사가 blank. NSIS 에서 레지스트리(EdgeUpdate pv) 확인 후 미설치 시 MicrosoftEdgeWebview2Setup.exe 를 silent 설치. package_win.ps1 이 부트스트래퍼를 자동 다운로드해 번들. (VC++ CRT/.NET-런타임 이슈는 CopyRuntime+vc_redist 로 기존에 이미 처리됨)</t>
+          <t>Rainbow PLA HS 프로파일 캘리브레이션 반영.</t>
         </is>
       </c>
     </row>
@@ -675,29 +675,29 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>G-code load</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>제품 버전 rc1 → rc2</t>
+          <t>OrcaForCubicon(1.4.1 등) 및 신규 1.5.0 gcode 로드 실패 수정 (patch 0008 회귀 대응)</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>gcode 로드 수정 + WebView2 런타임 준비 반영.</t>
+          <t>patch 0008 로 헤더를 '; generated by OrcaSlicer'로 바꾼 뒤, Config.cpp 의 로드 검증이 여전히 '; generated by OrcaForCubicon' 만 허용해 자기 파일조차 'Not a gcode file generated by OrcaForCubicon' 로 거부되던 문제. 검증에 '; generated by ' + SLIC3R_OFFICIAL_NAME('OrcaSlicer') 허용을 추가(patch 0008 갱신).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc1</t>
+          <t>1.5.1-rc2</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -707,29 +707,29 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>version / release</t>
+          <t>Installer / Runtime</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>기본 버전 1.5.0 → 1.5.1 (다음 개발 사이클 시작)</t>
+          <t>WebView2 Evergreen 런타임 조건부 설치 추가 (마법사 blank 방지)</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>GitHub v1.5.0 발행 후 v1.5.1 을 추가 발행하여, v1.5.0 실행 시 업데이트 알림 팝업이 정상 동작하는지 end-to-end 검증하기 위한 버전 업. release 빌드 시 '1.5.1' 로 태깅.</t>
+          <t>WebView2Loader.dll 만으로는 부족 — 클린 PC에 WebView2 런타임이 없으면 설정 마법사가 blank. NSIS 에서 레지스트리(EdgeUpdate pv) 확인 후 미설치 시 MicrosoftEdgeWebview2Setup.exe 를 silent 설치. package_win.ps1 이 부트스트래퍼를 자동 다운로드해 번들. (VC++ CRT/.NET-런타임 이슈는 CopyRuntime+vc_redist 로 기존에 이미 처리됨)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc5</t>
+          <t>1.5.1-rc2</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -739,29 +739,29 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Splash</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>다크모드 스플래시 로고에서 legacy 'style' 문구 제거</t>
+          <t>제품 버전 rc1 → rc2</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>splash_logo_dark.png 가 큐비콘 legacy 'style CUBICON' 로고였음(Style 시리즈는 OrcaForCubicon 미지원). light 로고 기반으로 흰색 CUBICON 텍스트 + 컬러 아이콘의 다크모드 전용 로고로 교체(2495→2125px).</t>
+          <t>gcode 로드 수정 + WebView2 런타임 준비 반영.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc5</t>
+          <t>1.5.1-rc1</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -776,24 +776,24 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>version / release</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc4 → rc5</t>
+          <t>기본 버전 1.5.0 → 1.5.1 (다음 개발 사이클 시작)</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>다크모드 스플래시 로고 수정 반영.</t>
+          <t>GitHub v1.5.0 발행 후 v1.5.1 을 추가 발행하여, v1.5.0 실행 시 업데이트 알림 팝업이 정상 동작하는지 end-to-end 검증하기 위한 버전 업. release 빌드 시 '1.5.1' 로 태깅.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc4</t>
+          <t>1.5.0-rc5</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -803,29 +803,29 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Build / Filament</t>
+          <t>Splash</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>테스트 전용 필라멘트 분리 (test 빌드=포함 / release 빌드=제외)</t>
+          <t>다크모드 스플래시 로고에서 legacy 'style' 문구 제거</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>cubicon/version/test_only_filaments.txt 매니페스트에 나열한 미검증 필라멘트를 release 빌드에서만 제거(cubicon/scripts/prune_test_filaments.ps1, build_win.ps1 -BuildType release 에서 호출). SSOT(cubicon/resources)는 전부 유지 → test 빌드는 모두 포함. 현재 test 전용: Cubicon Rainbow PLA HS, Cubicon TPU-HS(+fdm_filament_tpu). 검증 완료 시 매니페스트에서 해당 줄만 삭제하면 정식 승격.</t>
+          <t>splash_logo_dark.png 가 큐비콘 legacy 'style CUBICON' 로고였음(Style 시리즈는 OrcaForCubicon 미지원). light 로고 기반으로 흰색 CUBICON 텍스트 + 컬러 아이콘의 다크모드 전용 로고로 교체(2495→2125px).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc4</t>
+          <t>1.5.0-rc5</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -845,19 +845,19 @@
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc3 → rc4</t>
+          <t>제품 버전 rc4 → rc5</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>테스트/정식 필라멘트 분리 기능 반영.</t>
+          <t>다크모드 스플래시 로고 수정 반영.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc3</t>
+          <t>1.5.0-rc4</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -872,24 +872,24 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Update check</t>
+          <t>Build / Filament</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>OrcaForCubicon 전용 업데이트 알림 기능 (OrcaSlicer 기본 체크 비활성화)</t>
+          <t>테스트 전용 필라멘트 분리 (test 빌드=포함 / release 빌드=제외)</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>실행 시 GitHub 최신 릴리스(api.github.com/repos/Hyvision/OrcaForCubicon/releases/latest)를 조회해 제품버전 CUBI_ORCA_VERSION 과 비교, 새 정식 릴리스가 있으면 팝업 알림 → '다운로드' 시 브라우저로 릴리스 페이지 열기. 정식 릴리스만 대상(/releases/latest 가 draft·prerelease 자동 제외). OrcaSlicer 의 check_new_version_sf 는 시작·수동 '업데이트 확인' 메뉴 양쪽에서 check_new_version_cubicon 으로 대체. 기존 UpdateVersionDialog 재사용. (patch 0009) ※ 동작하려면 레포 public 전환 + GitHub Releases 발행 필요.</t>
+          <t>cubicon/version/test_only_filaments.txt 매니페스트에 나열한 미검증 필라멘트를 release 빌드에서만 제거(cubicon/scripts/prune_test_filaments.ps1, build_win.ps1 -BuildType release 에서 호출). SSOT(cubicon/resources)는 전부 유지 → test 빌드는 모두 포함. 현재 test 전용: Cubicon Rainbow PLA HS, Cubicon TPU-HS(+fdm_filament_tpu). 검증 완료 시 매니페스트에서 해당 줄만 삭제하면 정식 승격.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc3</t>
+          <t>1.5.0-rc4</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -909,19 +909,19 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc2 → rc3</t>
+          <t>제품 버전 rc3 → rc4</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>업데이트 알림 기능 추가 반영.</t>
+          <t>테스트/정식 필라멘트 분리 기능 반영.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc2</t>
+          <t>1.5.0-rc3</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -931,29 +931,29 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>G-code / Mainsail</t>
+          <t>Update check</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>G-code 헤더 슬라이서명·버전 정정 (Moonraker 메타데이터 파싱 복원)</t>
+          <t>OrcaForCubicon 전용 업데이트 알림 기능 (OrcaSlicer 기본 체크 비활성화)</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>header_slic3r_generated() 가 "OrcaForCubicon 2.4.2" → "OrcaSlicer &lt;제품버전&gt;" 로 변경. Moonraker/Mainsail 은 인식된 슬라이서명(OrcaSlicer 등)일 때만 슬라이싱 정보를 파싱함 → 기존엔 Unknown+정보 없음. 버전도 Orca 2.4.2 대신 재정의 제품버전 표기. Orca 자체 재파싱은 GCodeProcessor 의 "generated by OrcaSlicer" producer 태그로 유지. (patch 0008)</t>
+          <t>실행 시 GitHub 최신 릴리스(api.github.com/repos/Hyvision/OrcaForCubicon/releases/latest)를 조회해 제품버전 CUBI_ORCA_VERSION 과 비교, 새 정식 릴리스가 있으면 팝업 알림 → '다운로드' 시 브라우저로 릴리스 페이지 열기. 정식 릴리스만 대상(/releases/latest 가 draft·prerelease 자동 제외). OrcaSlicer 의 check_new_version_sf 는 시작·수동 '업데이트 확인' 메뉴 양쪽에서 check_new_version_cubicon 으로 대체. 기존 UpdateVersionDialog 재사용. (patch 0009) ※ 동작하려면 레포 public 전환 + GitHub Releases 발행 필요.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc2</t>
+          <t>1.5.0-rc3</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -963,22 +963,22 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>build_win.ps1</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>release / test 빌드 유형 옵션 추가</t>
+          <t>제품 버전 rc2 → rc3</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>-BuildType test|release (대화식 프롬프트 4번). release 는 버전의 -rc 접미사를 제거하여 splash·버전정보·About 대화상자·G-code 헤더·인스톨러명 모두에 반영. test 는 rc 유지. cubicon_version.txt(SSOT)를 빌드 중 임시 수정 후 finally 에서 원복.</t>
+          <t>업데이트 알림 기능 추가 반영.</t>
         </is>
       </c>
     </row>
@@ -995,22 +995,22 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>build_win.ps1</t>
+          <t>G-code / Mainsail</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>병렬 컴파일 잡을 메모리 기준으로도 제한 (-MemPerJobGB)</t>
+          <t>G-code 헤더 슬라이서명·버전 정정 (Moonraker 메타데이터 파싱 복원)</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>28코어/32GB 환경에서 CpuPercent 70%(=19잡)로 libslic3r PCH 컴파일 시 페이지파일 고갈(C3859/C1076/OS 1455) 발생. jobs = min(CPU 상한, floor((총RAM-4)/MemPerJobGB[기본3])) 로 제한하여 재발 방지.</t>
+          <t>header_slic3r_generated() 가 "OrcaForCubicon 2.4.2" → "OrcaSlicer &lt;제품버전&gt;" 로 변경. Moonraker/Mainsail 은 인식된 슬라이서명(OrcaSlicer 등)일 때만 슬라이싱 정보를 파싱함 → 기존엔 Unknown+정보 없음. 버전도 Orca 2.4.2 대신 재정의 제품버전 표기. Orca 자체 재파싱은 GCodeProcessor 의 "generated by OrcaSlicer" producer 태그로 유지. (patch 0008)</t>
         </is>
       </c>
     </row>
@@ -1027,29 +1027,29 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>build_win.ps1</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc1 → rc2</t>
+          <t>release / test 빌드 유형 옵션 추가</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>cubicon/version/cubicon_version.txt. 규칙: 매 수정마다 rc 1 증가(반영 여부 식별용).</t>
+          <t>-BuildType test|release (대화식 프롬프트 4번). release 는 버전의 -rc 접미사를 제거하여 splash·버전정보·About 대화상자·G-code 헤더·인스톨러명 모두에 반영. test 는 rc 유지. cubicon_version.txt(SSOT)를 빌드 중 임시 수정 후 finally 에서 원복.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc1</t>
+          <t>1.5.0-rc2</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -1059,29 +1059,29 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Machine profile</t>
+          <t>build_win.ps1</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>장비 Max Jerk 하향 (Bambu·Creality 기조: 고가감속·저저크)</t>
+          <t>병렬 컴파일 잡을 메모리 기준으로도 제한 (-MemPerJobGB)</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>xCeler-Plus/I/Mini 3종: X 20→5, Y 20→5, Z 20→2, E 20→2.5 mm/s. 캔틸레버 베드 편심 틸트로 레이어 중 Z가 상시 반전할 때 높은 Z 저크가 임펄스 진동→수직 벽면 잔상(ghosting)을 유발하던 문제 해결. 장비 프로파일 version → 1.5.0.</t>
+          <t>28코어/32GB 환경에서 CpuPercent 70%(=19잡)로 libslic3r PCH 컴파일 시 페이지파일 고갈(C3859/C1076/OS 1455) 발생. jobs = min(CPU 상한, floor((총RAM-4)/MemPerJobGB[기본3])) 로 제한하여 재발 방지.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc1</t>
+          <t>1.5.0-rc2</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1091,22 +1091,22 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Filament profile</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>신규 필라멘트: Cubicon TPU-HS</t>
+          <t>제품 버전 rc1 → rc2</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>isun3d TPU-HS(고속 TPU, Shore 95A) 추가. base + xCeler-I/Plus/Mini. fdm_filament_tpu 계열 베이스 신설. 초기값(노즐 230/230, 베드 50, 최대유량 5, 팬 100%) — 캘리브레이션 예정.</t>
+          <t>cubicon/version/cubicon_version.txt. 규칙: 매 수정마다 rc 1 증가(반영 여부 식별용).</t>
         </is>
       </c>
     </row>
@@ -1128,17 +1128,17 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Filament profile</t>
+          <t>Machine profile</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>신규 필라멘트: Cubicon Rainbow PLA HS</t>
+          <t>장비 Max Jerk 하향 (Bambu·Creality 기조: 고가감속·저저크)</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>한일 Rainbow PLA High Speed (Bambu PLA HS 유사). base + xCeler-I/Plus/Mini, Cubicon PLA @base 상속. 초기값(노즐 220/215, 베드 60, 최대유량 28, flow 0.98) — 캘리브레이션 예정.</t>
+          <t>xCeler-Plus/I/Mini 3종: X 20→5, Y 20→5, Z 20→2, E 20→2.5 mm/s. 캔틸레버 베드 편심 틸트로 레이어 중 Z가 상시 반전할 때 높은 Z 저크가 임펄스 진동→수직 벽면 잔상(ghosting)을 유발하던 문제 해결. 장비 프로파일 version → 1.5.0.</t>
         </is>
       </c>
     </row>
@@ -1155,20 +1155,84 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
+          <t>Feat</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Filament profile</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>신규 필라멘트: Cubicon TPU-HS</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>isun3d TPU-HS(고속 TPU, Shore 95A) 추가. base + xCeler-I/Plus/Mini. fdm_filament_tpu 계열 베이스 신설. 초기값(노즐 230/230, 베드 50, 최대유량 5, 팬 100%) — 캘리브레이션 예정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>1.5.0-rc1</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Feat</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Filament profile</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>신규 필라멘트: Cubicon Rainbow PLA HS</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>한일 Rainbow PLA High Speed (Bambu PLA HS 유사). base + xCeler-I/Plus/Mini, Cubicon PLA @base 상속. 초기값(노즐 220/215, 베드 60, 최대유량 28, flow 0.98) — 캘리브레이션 예정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>1.5.0-rc1</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
           <t>Chore</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D26" s="7" t="inlineStr">
         <is>
           <t>Profile package</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="E26" s="7" t="inlineStr">
         <is>
           <t>프로파일 패키지 버전 02.03.02.00 → 02.03.03.00</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="F26" s="7" t="inlineStr">
         <is>
           <t>Cubicon.json. 기설치 사용자에게 프로파일 갱신 전파를 위해 패키지 버전 상승 (신규 필라멘트·저크 반영).</t>
         </is>

</xml_diff>

<commit_message>
[cubicon] v1.5.1-rc5: fix build patch conflict (reset overlay to HEAD, not index)
build_win.ps1 reset the source with `git checkout -- src ...`, which resets the working
tree FROM the index. But `git apply --3way` stages patched files into the index on success,
so a prior build left old patched blobs staged; the next build reset to those and `git apply`
then conflicted whenever a patch had changed (e.g. after updating patch 0008):
  "Applied ... with conflicts / U src/libslic3r/utils.cpp / patch failed".
Changed to `git checkout HEAD -- src resources CMakeLists.txt version.inc` (resets BOTH the
index and the working tree to pristine HEAD every build). Verified: all 9 patches apply cleanly.

Bump product version rc4 -> rc5; update Excel release notes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
+++ b/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1.5.1-rc4</t>
+          <t>1.5.1-rc5</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -547,29 +547,29 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Process profile</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>정밀도(공차) 보정 기본 프로세스 반영 (전 재료 공통)</t>
+          <t>빌드 시 patch 0008 충돌(U src/libslic3r/utils.cpp) 수정</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>cubicon common @base: 코끼리발 보정 0.15→0.2 · 보정 레이어 2 · X-Y 구멍 보정 0.2 · X-Y 윤곽 보상 0.02 추가. resolution 0.012 · slice_closing 0.049 · EF density 100% · 정밀한 벽/정확한 Z · 원호맞춤 off 는 기존 일치. Rainbow PLA HS 공차 캘리브레이션 결과이며 공정 설정이라 전 재료에 공통 적용됨.</t>
+          <t>build_win.ps1 이 소스를 인덱스로 리셋('git checkout -- src')해, git apply --3way 가 staged 로 남긴 옛 패치본이 새 패치와 충돌하던 문제. 'git checkout HEAD -- ...'(인덱스+워크트리 모두 HEAD로 리셋)로 변경해 매 빌드 pristine 보장.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc4</t>
+          <t>1.5.1-rc5</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -589,19 +589,19 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc3 → rc4</t>
+          <t>제품 버전 rc4 → rc5</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>정밀도 공차 프로세스 반영.</t>
+          <t>빌드 스크립트 패치충돌 수정 반영.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>1.5.1-rc3</t>
+          <t>1.5.1-rc4</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -616,24 +616,24 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Filament profile</t>
+          <t>Process profile</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Rainbow PLA HS 캘리브레이션 확정값 반영</t>
+          <t>정밀도(공차) 보정 기본 프로세스 반영 (전 재료 공통)</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Cubicon Rainbow PLA HS @base: 최대 체적 속도 28→17 mm³/s(실측), Pressure Advance 0.03 신규 활성화. 온도(215/220)·베드(60)·유량비율(0.98)·후퇴(2mm 상속)는 캘리브레이션으로 적정 확인. 여전히 test-only. 상세: Rainbow PLA HS_ProfileUpdate_20260731_R0.pptx.</t>
+          <t>cubicon common @base: 코끼리발 보정 0.15→0.2 · 보정 레이어 2 · X-Y 구멍 보정 0.2 · X-Y 윤곽 보상 0.02 추가. resolution 0.012 · slice_closing 0.049 · EF density 100% · 정밀한 벽/정확한 Z · 원호맞춤 off 는 기존 일치. Rainbow PLA HS 공차 캘리브레이션 결과이며 공정 설정이라 전 재료에 공통 적용됨.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc3</t>
+          <t>1.5.1-rc4</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -653,76 +653,76 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc2 → rc3</t>
+          <t>제품 버전 rc3 → rc4</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Rainbow PLA HS 프로파일 캘리브레이션 반영.</t>
+          <t>정밀도 공차 프로세스 반영.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>1.5.1-rc2</t>
+          <t>1.5.1-rc3</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>G-code load</t>
+          <t>Filament profile</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>OrcaForCubicon(1.4.1 등) 및 신규 1.5.0 gcode 로드 실패 수정 (patch 0008 회귀 대응)</t>
+          <t>Rainbow PLA HS 캘리브레이션 확정값 반영</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>patch 0008 로 헤더를 '; generated by OrcaSlicer'로 바꾼 뒤, Config.cpp 의 로드 검증이 여전히 '; generated by OrcaForCubicon' 만 허용해 자기 파일조차 'Not a gcode file generated by OrcaForCubicon' 로 거부되던 문제. 검증에 '; generated by ' + SLIC3R_OFFICIAL_NAME('OrcaSlicer') 허용을 추가(patch 0008 갱신).</t>
+          <t>Cubicon Rainbow PLA HS @base: 최대 체적 속도 28→17 mm³/s(실측), Pressure Advance 0.03 신규 활성화. 온도(215/220)·베드(60)·유량비율(0.98)·후퇴(2mm 상속)는 캘리브레이션으로 적정 확인. 여전히 test-only. 상세: Rainbow PLA HS_ProfileUpdate_20260731_R0.pptx.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc2</t>
+          <t>1.5.1-rc3</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Installer / Runtime</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>WebView2 Evergreen 런타임 조건부 설치 추가 (마법사 blank 방지)</t>
+          <t>제품 버전 rc2 → rc3</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>WebView2Loader.dll 만으로는 부족 — 클린 PC에 WebView2 런타임이 없으면 설정 마법사가 blank. NSIS 에서 레지스트리(EdgeUpdate pv) 확인 후 미설치 시 MicrosoftEdgeWebview2Setup.exe 를 silent 설치. package_win.ps1 이 부트스트래퍼를 자동 다운로드해 번들. (VC++ CRT/.NET-런타임 이슈는 CopyRuntime+vc_redist 로 기존에 이미 처리됨)</t>
+          <t>Rainbow PLA HS 프로파일 캘리브레이션 반영.</t>
         </is>
       </c>
     </row>
@@ -739,29 +739,29 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>G-code load</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>제품 버전 rc1 → rc2</t>
+          <t>OrcaForCubicon(1.4.1 등) 및 신규 1.5.0 gcode 로드 실패 수정 (patch 0008 회귀 대응)</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>gcode 로드 수정 + WebView2 런타임 준비 반영.</t>
+          <t>patch 0008 로 헤더를 '; generated by OrcaSlicer'로 바꾼 뒤, Config.cpp 의 로드 검증이 여전히 '; generated by OrcaForCubicon' 만 허용해 자기 파일조차 'Not a gcode file generated by OrcaForCubicon' 로 거부되던 문제. 검증에 '; generated by ' + SLIC3R_OFFICIAL_NAME('OrcaSlicer') 허용을 추가(patch 0008 갱신).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc1</t>
+          <t>1.5.1-rc2</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -771,29 +771,29 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>version / release</t>
+          <t>Installer / Runtime</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>기본 버전 1.5.0 → 1.5.1 (다음 개발 사이클 시작)</t>
+          <t>WebView2 Evergreen 런타임 조건부 설치 추가 (마법사 blank 방지)</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>GitHub v1.5.0 발행 후 v1.5.1 을 추가 발행하여, v1.5.0 실행 시 업데이트 알림 팝업이 정상 동작하는지 end-to-end 검증하기 위한 버전 업. release 빌드 시 '1.5.1' 로 태깅.</t>
+          <t>WebView2Loader.dll 만으로는 부족 — 클린 PC에 WebView2 런타임이 없으면 설정 마법사가 blank. NSIS 에서 레지스트리(EdgeUpdate pv) 확인 후 미설치 시 MicrosoftEdgeWebview2Setup.exe 를 silent 설치. package_win.ps1 이 부트스트래퍼를 자동 다운로드해 번들. (VC++ CRT/.NET-런타임 이슈는 CopyRuntime+vc_redist 로 기존에 이미 처리됨)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc5</t>
+          <t>1.5.1-rc2</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -803,29 +803,29 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Splash</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>다크모드 스플래시 로고에서 legacy 'style' 문구 제거</t>
+          <t>제품 버전 rc1 → rc2</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>splash_logo_dark.png 가 큐비콘 legacy 'style CUBICON' 로고였음(Style 시리즈는 OrcaForCubicon 미지원). light 로고 기반으로 흰색 CUBICON 텍스트 + 컬러 아이콘의 다크모드 전용 로고로 교체(2495→2125px).</t>
+          <t>gcode 로드 수정 + WebView2 런타임 준비 반영.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc5</t>
+          <t>1.5.1-rc1</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -840,24 +840,24 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>version / release</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc4 → rc5</t>
+          <t>기본 버전 1.5.0 → 1.5.1 (다음 개발 사이클 시작)</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>다크모드 스플래시 로고 수정 반영.</t>
+          <t>GitHub v1.5.0 발행 후 v1.5.1 을 추가 발행하여, v1.5.0 실행 시 업데이트 알림 팝업이 정상 동작하는지 end-to-end 검증하기 위한 버전 업. release 빌드 시 '1.5.1' 로 태깅.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc4</t>
+          <t>1.5.0-rc5</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -867,29 +867,29 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Build / Filament</t>
+          <t>Splash</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>테스트 전용 필라멘트 분리 (test 빌드=포함 / release 빌드=제외)</t>
+          <t>다크모드 스플래시 로고에서 legacy 'style' 문구 제거</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>cubicon/version/test_only_filaments.txt 매니페스트에 나열한 미검증 필라멘트를 release 빌드에서만 제거(cubicon/scripts/prune_test_filaments.ps1, build_win.ps1 -BuildType release 에서 호출). SSOT(cubicon/resources)는 전부 유지 → test 빌드는 모두 포함. 현재 test 전용: Cubicon Rainbow PLA HS, Cubicon TPU-HS(+fdm_filament_tpu). 검증 완료 시 매니페스트에서 해당 줄만 삭제하면 정식 승격.</t>
+          <t>splash_logo_dark.png 가 큐비콘 legacy 'style CUBICON' 로고였음(Style 시리즈는 OrcaForCubicon 미지원). light 로고 기반으로 흰색 CUBICON 텍스트 + 컬러 아이콘의 다크모드 전용 로고로 교체(2495→2125px).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc4</t>
+          <t>1.5.0-rc5</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -909,19 +909,19 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc3 → rc4</t>
+          <t>제품 버전 rc4 → rc5</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>테스트/정식 필라멘트 분리 기능 반영.</t>
+          <t>다크모드 스플래시 로고 수정 반영.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc3</t>
+          <t>1.5.0-rc4</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -936,24 +936,24 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Update check</t>
+          <t>Build / Filament</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>OrcaForCubicon 전용 업데이트 알림 기능 (OrcaSlicer 기본 체크 비활성화)</t>
+          <t>테스트 전용 필라멘트 분리 (test 빌드=포함 / release 빌드=제외)</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>실행 시 GitHub 최신 릴리스(api.github.com/repos/Hyvision/OrcaForCubicon/releases/latest)를 조회해 제품버전 CUBI_ORCA_VERSION 과 비교, 새 정식 릴리스가 있으면 팝업 알림 → '다운로드' 시 브라우저로 릴리스 페이지 열기. 정식 릴리스만 대상(/releases/latest 가 draft·prerelease 자동 제외). OrcaSlicer 의 check_new_version_sf 는 시작·수동 '업데이트 확인' 메뉴 양쪽에서 check_new_version_cubicon 으로 대체. 기존 UpdateVersionDialog 재사용. (patch 0009) ※ 동작하려면 레포 public 전환 + GitHub Releases 발행 필요.</t>
+          <t>cubicon/version/test_only_filaments.txt 매니페스트에 나열한 미검증 필라멘트를 release 빌드에서만 제거(cubicon/scripts/prune_test_filaments.ps1, build_win.ps1 -BuildType release 에서 호출). SSOT(cubicon/resources)는 전부 유지 → test 빌드는 모두 포함. 현재 test 전용: Cubicon Rainbow PLA HS, Cubicon TPU-HS(+fdm_filament_tpu). 검증 완료 시 매니페스트에서 해당 줄만 삭제하면 정식 승격.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc3</t>
+          <t>1.5.0-rc4</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -973,19 +973,19 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc2 → rc3</t>
+          <t>제품 버전 rc3 → rc4</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>업데이트 알림 기능 추가 반영.</t>
+          <t>테스트/정식 필라멘트 분리 기능 반영.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc2</t>
+          <t>1.5.0-rc3</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -995,29 +995,29 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>G-code / Mainsail</t>
+          <t>Update check</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>G-code 헤더 슬라이서명·버전 정정 (Moonraker 메타데이터 파싱 복원)</t>
+          <t>OrcaForCubicon 전용 업데이트 알림 기능 (OrcaSlicer 기본 체크 비활성화)</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>header_slic3r_generated() 가 "OrcaForCubicon 2.4.2" → "OrcaSlicer &lt;제품버전&gt;" 로 변경. Moonraker/Mainsail 은 인식된 슬라이서명(OrcaSlicer 등)일 때만 슬라이싱 정보를 파싱함 → 기존엔 Unknown+정보 없음. 버전도 Orca 2.4.2 대신 재정의 제품버전 표기. Orca 자체 재파싱은 GCodeProcessor 의 "generated by OrcaSlicer" producer 태그로 유지. (patch 0008)</t>
+          <t>실행 시 GitHub 최신 릴리스(api.github.com/repos/Hyvision/OrcaForCubicon/releases/latest)를 조회해 제품버전 CUBI_ORCA_VERSION 과 비교, 새 정식 릴리스가 있으면 팝업 알림 → '다운로드' 시 브라우저로 릴리스 페이지 열기. 정식 릴리스만 대상(/releases/latest 가 draft·prerelease 자동 제외). OrcaSlicer 의 check_new_version_sf 는 시작·수동 '업데이트 확인' 메뉴 양쪽에서 check_new_version_cubicon 으로 대체. 기존 UpdateVersionDialog 재사용. (patch 0009) ※ 동작하려면 레포 public 전환 + GitHub Releases 발행 필요.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc2</t>
+          <t>1.5.0-rc3</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -1027,22 +1027,22 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>build_win.ps1</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>release / test 빌드 유형 옵션 추가</t>
+          <t>제품 버전 rc2 → rc3</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>-BuildType test|release (대화식 프롬프트 4번). release 는 버전의 -rc 접미사를 제거하여 splash·버전정보·About 대화상자·G-code 헤더·인스톨러명 모두에 반영. test 는 rc 유지. cubicon_version.txt(SSOT)를 빌드 중 임시 수정 후 finally 에서 원복.</t>
+          <t>업데이트 알림 기능 추가 반영.</t>
         </is>
       </c>
     </row>
@@ -1059,22 +1059,22 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>build_win.ps1</t>
+          <t>G-code / Mainsail</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>병렬 컴파일 잡을 메모리 기준으로도 제한 (-MemPerJobGB)</t>
+          <t>G-code 헤더 슬라이서명·버전 정정 (Moonraker 메타데이터 파싱 복원)</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>28코어/32GB 환경에서 CpuPercent 70%(=19잡)로 libslic3r PCH 컴파일 시 페이지파일 고갈(C3859/C1076/OS 1455) 발생. jobs = min(CPU 상한, floor((총RAM-4)/MemPerJobGB[기본3])) 로 제한하여 재발 방지.</t>
+          <t>header_slic3r_generated() 가 "OrcaForCubicon 2.4.2" → "OrcaSlicer &lt;제품버전&gt;" 로 변경. Moonraker/Mainsail 은 인식된 슬라이서명(OrcaSlicer 등)일 때만 슬라이싱 정보를 파싱함 → 기존엔 Unknown+정보 없음. 버전도 Orca 2.4.2 대신 재정의 제품버전 표기. Orca 자체 재파싱은 GCodeProcessor 의 "generated by OrcaSlicer" producer 태그로 유지. (patch 0008)</t>
         </is>
       </c>
     </row>
@@ -1091,29 +1091,29 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>build_win.ps1</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc1 → rc2</t>
+          <t>release / test 빌드 유형 옵션 추가</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>cubicon/version/cubicon_version.txt. 규칙: 매 수정마다 rc 1 증가(반영 여부 식별용).</t>
+          <t>-BuildType test|release (대화식 프롬프트 4번). release 는 버전의 -rc 접미사를 제거하여 splash·버전정보·About 대화상자·G-code 헤더·인스톨러명 모두에 반영. test 는 rc 유지. cubicon_version.txt(SSOT)를 빌드 중 임시 수정 후 finally 에서 원복.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc1</t>
+          <t>1.5.0-rc2</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -1123,29 +1123,29 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Machine profile</t>
+          <t>build_win.ps1</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>장비 Max Jerk 하향 (Bambu·Creality 기조: 고가감속·저저크)</t>
+          <t>병렬 컴파일 잡을 메모리 기준으로도 제한 (-MemPerJobGB)</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>xCeler-Plus/I/Mini 3종: X 20→5, Y 20→5, Z 20→2, E 20→2.5 mm/s. 캔틸레버 베드 편심 틸트로 레이어 중 Z가 상시 반전할 때 높은 Z 저크가 임펄스 진동→수직 벽면 잔상(ghosting)을 유발하던 문제 해결. 장비 프로파일 version → 1.5.0.</t>
+          <t>28코어/32GB 환경에서 CpuPercent 70%(=19잡)로 libslic3r PCH 컴파일 시 페이지파일 고갈(C3859/C1076/OS 1455) 발생. jobs = min(CPU 상한, floor((총RAM-4)/MemPerJobGB[기본3])) 로 제한하여 재발 방지.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc1</t>
+          <t>1.5.0-rc2</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1155,22 +1155,22 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Filament profile</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>신규 필라멘트: Cubicon TPU-HS</t>
+          <t>제품 버전 rc1 → rc2</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>isun3d TPU-HS(고속 TPU, Shore 95A) 추가. base + xCeler-I/Plus/Mini. fdm_filament_tpu 계열 베이스 신설. 초기값(노즐 230/230, 베드 50, 최대유량 5, 팬 100%) — 캘리브레이션 예정.</t>
+          <t>cubicon/version/cubicon_version.txt. 규칙: 매 수정마다 rc 1 증가(반영 여부 식별용).</t>
         </is>
       </c>
     </row>
@@ -1192,17 +1192,17 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Filament profile</t>
+          <t>Machine profile</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>신규 필라멘트: Cubicon Rainbow PLA HS</t>
+          <t>장비 Max Jerk 하향 (Bambu·Creality 기조: 고가감속·저저크)</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>한일 Rainbow PLA High Speed (Bambu PLA HS 유사). base + xCeler-I/Plus/Mini, Cubicon PLA @base 상속. 초기값(노즐 220/215, 베드 60, 최대유량 28, flow 0.98) — 캘리브레이션 예정.</t>
+          <t>xCeler-Plus/I/Mini 3종: X 20→5, Y 20→5, Z 20→2, E 20→2.5 mm/s. 캔틸레버 베드 편심 틸트로 레이어 중 Z가 상시 반전할 때 높은 Z 저크가 임펄스 진동→수직 벽면 잔상(ghosting)을 유발하던 문제 해결. 장비 프로파일 version → 1.5.0.</t>
         </is>
       </c>
     </row>
@@ -1219,20 +1219,84 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
+          <t>Feat</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Filament profile</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>신규 필라멘트: Cubicon TPU-HS</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>isun3d TPU-HS(고속 TPU, Shore 95A) 추가. base + xCeler-I/Plus/Mini. fdm_filament_tpu 계열 베이스 신설. 초기값(노즐 230/230, 베드 50, 최대유량 5, 팬 100%) — 캘리브레이션 예정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>1.5.0-rc1</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Feat</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Filament profile</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>신규 필라멘트: Cubicon Rainbow PLA HS</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>한일 Rainbow PLA High Speed (Bambu PLA HS 유사). base + xCeler-I/Plus/Mini, Cubicon PLA @base 상속. 초기값(노즐 220/215, 베드 60, 최대유량 28, flow 0.98) — 캘리브레이션 예정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>1.5.0-rc1</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
           <t>Chore</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D28" s="7" t="inlineStr">
         <is>
           <t>Profile package</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="E28" s="7" t="inlineStr">
         <is>
           <t>프로파일 패키지 버전 02.03.02.00 → 02.03.03.00</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
+      <c r="F28" s="7" t="inlineStr">
         <is>
           <t>Cubicon.json. 기설치 사용자에게 프로파일 갱신 전파를 위해 패키지 버전 상승 (신규 필라멘트·저크 반영).</t>
         </is>

</xml_diff>

<commit_message>
[cubicon] v1.5.1-rc6: change support/raft/overhang defaults in base process
cubicon common @base (shared by all Cubicon processes -> applies to every material):
- enable_support 0 -> 1
- support_on_build_plate_only 1 -> 0
- support_threshold_angle 15 -> 30
- support_type normal(auto) -> tree(auto)
- raft_contact_distance 0.1 -> 0.2 (was inherited)
- raft_layers 0 -> 3
- detect_overhang_wall 0 -> 1

Bump product version rc5 -> rc6; update Excel release notes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
+++ b/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1.5.1-rc5</t>
+          <t>1.5.1-rc6</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -547,29 +547,29 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Process profile</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>빌드 시 patch 0008 충돌(U src/libslic3r/utils.cpp) 수정</t>
+          <t>서포트·라프트·오버행 기본값 변경 (기본 프로세스, 전 재료 공통)</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>build_win.ps1 이 소스를 인덱스로 리셋('git checkout -- src')해, git apply --3way 가 staged 로 남긴 옛 패치본이 새 패치와 충돌하던 문제. 'git checkout HEAD -- ...'(인덱스+워크트리 모두 HEAD로 리셋)로 변경해 매 빌드 pristine 보장.</t>
+          <t>cubicon common @base: 서포트 사용 off→on, 빌드플레이트에만 on→off, 임계각 15→30, 유형 normal(auto)→tree(auto), 라프트 접점 Z 0.1→0.2, 라프트 레이어 0→3, 오버행 벽 감지 off→on.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc5</t>
+          <t>1.5.1-rc6</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -589,19 +589,19 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc4 → rc5</t>
+          <t>제품 버전 rc5 → rc6</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>빌드 스크립트 패치충돌 수정 반영.</t>
+          <t>서포트 옵션 변경 반영.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>1.5.1-rc4</t>
+          <t>1.5.1-rc5</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -611,29 +611,29 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Process profile</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>정밀도(공차) 보정 기본 프로세스 반영 (전 재료 공통)</t>
+          <t>빌드 시 patch 0008 충돌(U src/libslic3r/utils.cpp) 수정</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>cubicon common @base: 코끼리발 보정 0.15→0.2 · 보정 레이어 2 · X-Y 구멍 보정 0.2 · X-Y 윤곽 보상 0.02 추가. resolution 0.012 · slice_closing 0.049 · EF density 100% · 정밀한 벽/정확한 Z · 원호맞춤 off 는 기존 일치. Rainbow PLA HS 공차 캘리브레이션 결과이며 공정 설정이라 전 재료에 공통 적용됨.</t>
+          <t>build_win.ps1 이 소스를 인덱스로 리셋('git checkout -- src')해, git apply --3way 가 staged 로 남긴 옛 패치본이 새 패치와 충돌하던 문제. 'git checkout HEAD -- ...'(인덱스+워크트리 모두 HEAD로 리셋)로 변경해 매 빌드 pristine 보장.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc4</t>
+          <t>1.5.1-rc5</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -653,19 +653,19 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc3 → rc4</t>
+          <t>제품 버전 rc4 → rc5</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>정밀도 공차 프로세스 반영.</t>
+          <t>빌드 스크립트 패치충돌 수정 반영.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>1.5.1-rc3</t>
+          <t>1.5.1-rc4</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -680,24 +680,24 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Filament profile</t>
+          <t>Process profile</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Rainbow PLA HS 캘리브레이션 확정값 반영</t>
+          <t>정밀도(공차) 보정 기본 프로세스 반영 (전 재료 공통)</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Cubicon Rainbow PLA HS @base: 최대 체적 속도 28→17 mm³/s(실측), Pressure Advance 0.03 신규 활성화. 온도(215/220)·베드(60)·유량비율(0.98)·후퇴(2mm 상속)는 캘리브레이션으로 적정 확인. 여전히 test-only. 상세: Rainbow PLA HS_ProfileUpdate_20260731_R0.pptx.</t>
+          <t>cubicon common @base: 코끼리발 보정 0.15→0.2 · 보정 레이어 2 · X-Y 구멍 보정 0.2 · X-Y 윤곽 보상 0.02 추가. resolution 0.012 · slice_closing 0.049 · EF density 100% · 정밀한 벽/정확한 Z · 원호맞춤 off 는 기존 일치. Rainbow PLA HS 공차 캘리브레이션 결과이며 공정 설정이라 전 재료에 공통 적용됨.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc3</t>
+          <t>1.5.1-rc4</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -717,76 +717,76 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc2 → rc3</t>
+          <t>제품 버전 rc3 → rc4</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Rainbow PLA HS 프로파일 캘리브레이션 반영.</t>
+          <t>정밀도 공차 프로세스 반영.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>1.5.1-rc2</t>
+          <t>1.5.1-rc3</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>G-code load</t>
+          <t>Filament profile</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>OrcaForCubicon(1.4.1 등) 및 신규 1.5.0 gcode 로드 실패 수정 (patch 0008 회귀 대응)</t>
+          <t>Rainbow PLA HS 캘리브레이션 확정값 반영</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>patch 0008 로 헤더를 '; generated by OrcaSlicer'로 바꾼 뒤, Config.cpp 의 로드 검증이 여전히 '; generated by OrcaForCubicon' 만 허용해 자기 파일조차 'Not a gcode file generated by OrcaForCubicon' 로 거부되던 문제. 검증에 '; generated by ' + SLIC3R_OFFICIAL_NAME('OrcaSlicer') 허용을 추가(patch 0008 갱신).</t>
+          <t>Cubicon Rainbow PLA HS @base: 최대 체적 속도 28→17 mm³/s(실측), Pressure Advance 0.03 신규 활성화. 온도(215/220)·베드(60)·유량비율(0.98)·후퇴(2mm 상속)는 캘리브레이션으로 적정 확인. 여전히 test-only. 상세: Rainbow PLA HS_ProfileUpdate_20260731_R0.pptx.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc2</t>
+          <t>1.5.1-rc3</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Installer / Runtime</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>WebView2 Evergreen 런타임 조건부 설치 추가 (마법사 blank 방지)</t>
+          <t>제품 버전 rc2 → rc3</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>WebView2Loader.dll 만으로는 부족 — 클린 PC에 WebView2 런타임이 없으면 설정 마법사가 blank. NSIS 에서 레지스트리(EdgeUpdate pv) 확인 후 미설치 시 MicrosoftEdgeWebview2Setup.exe 를 silent 설치. package_win.ps1 이 부트스트래퍼를 자동 다운로드해 번들. (VC++ CRT/.NET-런타임 이슈는 CopyRuntime+vc_redist 로 기존에 이미 처리됨)</t>
+          <t>Rainbow PLA HS 프로파일 캘리브레이션 반영.</t>
         </is>
       </c>
     </row>
@@ -803,29 +803,29 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>G-code load</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>제품 버전 rc1 → rc2</t>
+          <t>OrcaForCubicon(1.4.1 등) 및 신규 1.5.0 gcode 로드 실패 수정 (patch 0008 회귀 대응)</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>gcode 로드 수정 + WebView2 런타임 준비 반영.</t>
+          <t>patch 0008 로 헤더를 '; generated by OrcaSlicer'로 바꾼 뒤, Config.cpp 의 로드 검증이 여전히 '; generated by OrcaForCubicon' 만 허용해 자기 파일조차 'Not a gcode file generated by OrcaForCubicon' 로 거부되던 문제. 검증에 '; generated by ' + SLIC3R_OFFICIAL_NAME('OrcaSlicer') 허용을 추가(patch 0008 갱신).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc1</t>
+          <t>1.5.1-rc2</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -835,29 +835,29 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>version / release</t>
+          <t>Installer / Runtime</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>기본 버전 1.5.0 → 1.5.1 (다음 개발 사이클 시작)</t>
+          <t>WebView2 Evergreen 런타임 조건부 설치 추가 (마법사 blank 방지)</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>GitHub v1.5.0 발행 후 v1.5.1 을 추가 발행하여, v1.5.0 실행 시 업데이트 알림 팝업이 정상 동작하는지 end-to-end 검증하기 위한 버전 업. release 빌드 시 '1.5.1' 로 태깅.</t>
+          <t>WebView2Loader.dll 만으로는 부족 — 클린 PC에 WebView2 런타임이 없으면 설정 마법사가 blank. NSIS 에서 레지스트리(EdgeUpdate pv) 확인 후 미설치 시 MicrosoftEdgeWebview2Setup.exe 를 silent 설치. package_win.ps1 이 부트스트래퍼를 자동 다운로드해 번들. (VC++ CRT/.NET-런타임 이슈는 CopyRuntime+vc_redist 로 기존에 이미 처리됨)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc5</t>
+          <t>1.5.1-rc2</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -867,29 +867,29 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Splash</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>다크모드 스플래시 로고에서 legacy 'style' 문구 제거</t>
+          <t>제품 버전 rc1 → rc2</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>splash_logo_dark.png 가 큐비콘 legacy 'style CUBICON' 로고였음(Style 시리즈는 OrcaForCubicon 미지원). light 로고 기반으로 흰색 CUBICON 텍스트 + 컬러 아이콘의 다크모드 전용 로고로 교체(2495→2125px).</t>
+          <t>gcode 로드 수정 + WebView2 런타임 준비 반영.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc5</t>
+          <t>1.5.1-rc1</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -904,24 +904,24 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>version / release</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc4 → rc5</t>
+          <t>기본 버전 1.5.0 → 1.5.1 (다음 개발 사이클 시작)</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>다크모드 스플래시 로고 수정 반영.</t>
+          <t>GitHub v1.5.0 발행 후 v1.5.1 을 추가 발행하여, v1.5.0 실행 시 업데이트 알림 팝업이 정상 동작하는지 end-to-end 검증하기 위한 버전 업. release 빌드 시 '1.5.1' 로 태깅.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc4</t>
+          <t>1.5.0-rc5</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -931,29 +931,29 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Build / Filament</t>
+          <t>Splash</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>테스트 전용 필라멘트 분리 (test 빌드=포함 / release 빌드=제외)</t>
+          <t>다크모드 스플래시 로고에서 legacy 'style' 문구 제거</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>cubicon/version/test_only_filaments.txt 매니페스트에 나열한 미검증 필라멘트를 release 빌드에서만 제거(cubicon/scripts/prune_test_filaments.ps1, build_win.ps1 -BuildType release 에서 호출). SSOT(cubicon/resources)는 전부 유지 → test 빌드는 모두 포함. 현재 test 전용: Cubicon Rainbow PLA HS, Cubicon TPU-HS(+fdm_filament_tpu). 검증 완료 시 매니페스트에서 해당 줄만 삭제하면 정식 승격.</t>
+          <t>splash_logo_dark.png 가 큐비콘 legacy 'style CUBICON' 로고였음(Style 시리즈는 OrcaForCubicon 미지원). light 로고 기반으로 흰색 CUBICON 텍스트 + 컬러 아이콘의 다크모드 전용 로고로 교체(2495→2125px).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc4</t>
+          <t>1.5.0-rc5</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -973,19 +973,19 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc3 → rc4</t>
+          <t>제품 버전 rc4 → rc5</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>테스트/정식 필라멘트 분리 기능 반영.</t>
+          <t>다크모드 스플래시 로고 수정 반영.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc3</t>
+          <t>1.5.0-rc4</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1000,24 +1000,24 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Update check</t>
+          <t>Build / Filament</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>OrcaForCubicon 전용 업데이트 알림 기능 (OrcaSlicer 기본 체크 비활성화)</t>
+          <t>테스트 전용 필라멘트 분리 (test 빌드=포함 / release 빌드=제외)</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>실행 시 GitHub 최신 릴리스(api.github.com/repos/Hyvision/OrcaForCubicon/releases/latest)를 조회해 제품버전 CUBI_ORCA_VERSION 과 비교, 새 정식 릴리스가 있으면 팝업 알림 → '다운로드' 시 브라우저로 릴리스 페이지 열기. 정식 릴리스만 대상(/releases/latest 가 draft·prerelease 자동 제외). OrcaSlicer 의 check_new_version_sf 는 시작·수동 '업데이트 확인' 메뉴 양쪽에서 check_new_version_cubicon 으로 대체. 기존 UpdateVersionDialog 재사용. (patch 0009) ※ 동작하려면 레포 public 전환 + GitHub Releases 발행 필요.</t>
+          <t>cubicon/version/test_only_filaments.txt 매니페스트에 나열한 미검증 필라멘트를 release 빌드에서만 제거(cubicon/scripts/prune_test_filaments.ps1, build_win.ps1 -BuildType release 에서 호출). SSOT(cubicon/resources)는 전부 유지 → test 빌드는 모두 포함. 현재 test 전용: Cubicon Rainbow PLA HS, Cubicon TPU-HS(+fdm_filament_tpu). 검증 완료 시 매니페스트에서 해당 줄만 삭제하면 정식 승격.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc3</t>
+          <t>1.5.0-rc4</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -1037,19 +1037,19 @@
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc2 → rc3</t>
+          <t>제품 버전 rc3 → rc4</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>업데이트 알림 기능 추가 반영.</t>
+          <t>테스트/정식 필라멘트 분리 기능 반영.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc2</t>
+          <t>1.5.0-rc3</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -1059,29 +1059,29 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>G-code / Mainsail</t>
+          <t>Update check</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>G-code 헤더 슬라이서명·버전 정정 (Moonraker 메타데이터 파싱 복원)</t>
+          <t>OrcaForCubicon 전용 업데이트 알림 기능 (OrcaSlicer 기본 체크 비활성화)</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>header_slic3r_generated() 가 "OrcaForCubicon 2.4.2" → "OrcaSlicer &lt;제품버전&gt;" 로 변경. Moonraker/Mainsail 은 인식된 슬라이서명(OrcaSlicer 등)일 때만 슬라이싱 정보를 파싱함 → 기존엔 Unknown+정보 없음. 버전도 Orca 2.4.2 대신 재정의 제품버전 표기. Orca 자체 재파싱은 GCodeProcessor 의 "generated by OrcaSlicer" producer 태그로 유지. (patch 0008)</t>
+          <t>실행 시 GitHub 최신 릴리스(api.github.com/repos/Hyvision/OrcaForCubicon/releases/latest)를 조회해 제품버전 CUBI_ORCA_VERSION 과 비교, 새 정식 릴리스가 있으면 팝업 알림 → '다운로드' 시 브라우저로 릴리스 페이지 열기. 정식 릴리스만 대상(/releases/latest 가 draft·prerelease 자동 제외). OrcaSlicer 의 check_new_version_sf 는 시작·수동 '업데이트 확인' 메뉴 양쪽에서 check_new_version_cubicon 으로 대체. 기존 UpdateVersionDialog 재사용. (patch 0009) ※ 동작하려면 레포 public 전환 + GitHub Releases 발행 필요.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc2</t>
+          <t>1.5.0-rc3</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1091,22 +1091,22 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>build_win.ps1</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>release / test 빌드 유형 옵션 추가</t>
+          <t>제품 버전 rc2 → rc3</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>-BuildType test|release (대화식 프롬프트 4번). release 는 버전의 -rc 접미사를 제거하여 splash·버전정보·About 대화상자·G-code 헤더·인스톨러명 모두에 반영. test 는 rc 유지. cubicon_version.txt(SSOT)를 빌드 중 임시 수정 후 finally 에서 원복.</t>
+          <t>업데이트 알림 기능 추가 반영.</t>
         </is>
       </c>
     </row>
@@ -1123,22 +1123,22 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>build_win.ps1</t>
+          <t>G-code / Mainsail</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>병렬 컴파일 잡을 메모리 기준으로도 제한 (-MemPerJobGB)</t>
+          <t>G-code 헤더 슬라이서명·버전 정정 (Moonraker 메타데이터 파싱 복원)</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>28코어/32GB 환경에서 CpuPercent 70%(=19잡)로 libslic3r PCH 컴파일 시 페이지파일 고갈(C3859/C1076/OS 1455) 발생. jobs = min(CPU 상한, floor((총RAM-4)/MemPerJobGB[기본3])) 로 제한하여 재발 방지.</t>
+          <t>header_slic3r_generated() 가 "OrcaForCubicon 2.4.2" → "OrcaSlicer &lt;제품버전&gt;" 로 변경. Moonraker/Mainsail 은 인식된 슬라이서명(OrcaSlicer 등)일 때만 슬라이싱 정보를 파싱함 → 기존엔 Unknown+정보 없음. 버전도 Orca 2.4.2 대신 재정의 제품버전 표기. Orca 자체 재파싱은 GCodeProcessor 의 "generated by OrcaSlicer" producer 태그로 유지. (patch 0008)</t>
         </is>
       </c>
     </row>
@@ -1155,29 +1155,29 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>build_win.ps1</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc1 → rc2</t>
+          <t>release / test 빌드 유형 옵션 추가</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>cubicon/version/cubicon_version.txt. 규칙: 매 수정마다 rc 1 증가(반영 여부 식별용).</t>
+          <t>-BuildType test|release (대화식 프롬프트 4번). release 는 버전의 -rc 접미사를 제거하여 splash·버전정보·About 대화상자·G-code 헤더·인스톨러명 모두에 반영. test 는 rc 유지. cubicon_version.txt(SSOT)를 빌드 중 임시 수정 후 finally 에서 원복.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc1</t>
+          <t>1.5.0-rc2</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -1187,29 +1187,29 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Machine profile</t>
+          <t>build_win.ps1</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>장비 Max Jerk 하향 (Bambu·Creality 기조: 고가감속·저저크)</t>
+          <t>병렬 컴파일 잡을 메모리 기준으로도 제한 (-MemPerJobGB)</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>xCeler-Plus/I/Mini 3종: X 20→5, Y 20→5, Z 20→2, E 20→2.5 mm/s. 캔틸레버 베드 편심 틸트로 레이어 중 Z가 상시 반전할 때 높은 Z 저크가 임펄스 진동→수직 벽면 잔상(ghosting)을 유발하던 문제 해결. 장비 프로파일 version → 1.5.0.</t>
+          <t>28코어/32GB 환경에서 CpuPercent 70%(=19잡)로 libslic3r PCH 컴파일 시 페이지파일 고갈(C3859/C1076/OS 1455) 발생. jobs = min(CPU 상한, floor((총RAM-4)/MemPerJobGB[기본3])) 로 제한하여 재발 방지.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc1</t>
+          <t>1.5.0-rc2</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1219,22 +1219,22 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Filament profile</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>신규 필라멘트: Cubicon TPU-HS</t>
+          <t>제품 버전 rc1 → rc2</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>isun3d TPU-HS(고속 TPU, Shore 95A) 추가. base + xCeler-I/Plus/Mini. fdm_filament_tpu 계열 베이스 신설. 초기값(노즐 230/230, 베드 50, 최대유량 5, 팬 100%) — 캘리브레이션 예정.</t>
+          <t>cubicon/version/cubicon_version.txt. 규칙: 매 수정마다 rc 1 증가(반영 여부 식별용).</t>
         </is>
       </c>
     </row>
@@ -1256,17 +1256,17 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Filament profile</t>
+          <t>Machine profile</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>신규 필라멘트: Cubicon Rainbow PLA HS</t>
+          <t>장비 Max Jerk 하향 (Bambu·Creality 기조: 고가감속·저저크)</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>한일 Rainbow PLA High Speed (Bambu PLA HS 유사). base + xCeler-I/Plus/Mini, Cubicon PLA @base 상속. 초기값(노즐 220/215, 베드 60, 최대유량 28, flow 0.98) — 캘리브레이션 예정.</t>
+          <t>xCeler-Plus/I/Mini 3종: X 20→5, Y 20→5, Z 20→2, E 20→2.5 mm/s. 캔틸레버 베드 편심 틸트로 레이어 중 Z가 상시 반전할 때 높은 Z 저크가 임펄스 진동→수직 벽면 잔상(ghosting)을 유발하던 문제 해결. 장비 프로파일 version → 1.5.0.</t>
         </is>
       </c>
     </row>
@@ -1283,20 +1283,84 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
+          <t>Feat</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Filament profile</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>신규 필라멘트: Cubicon TPU-HS</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>isun3d TPU-HS(고속 TPU, Shore 95A) 추가. base + xCeler-I/Plus/Mini. fdm_filament_tpu 계열 베이스 신설. 초기값(노즐 230/230, 베드 50, 최대유량 5, 팬 100%) — 캘리브레이션 예정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>1.5.0-rc1</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Feat</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Filament profile</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>신규 필라멘트: Cubicon Rainbow PLA HS</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>한일 Rainbow PLA High Speed (Bambu PLA HS 유사). base + xCeler-I/Plus/Mini, Cubicon PLA @base 상속. 초기값(노즐 220/215, 베드 60, 최대유량 28, flow 0.98) — 캘리브레이션 예정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>1.5.0-rc1</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
           <t>Chore</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D30" s="7" t="inlineStr">
         <is>
           <t>Profile package</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E30" s="7" t="inlineStr">
         <is>
           <t>프로파일 패키지 버전 02.03.02.00 → 02.03.03.00</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
+      <c r="F30" s="7" t="inlineStr">
         <is>
           <t>Cubicon.json. 기설치 사용자에게 프로파일 갱신 전파를 위해 패키지 버전 상승 (신규 필라멘트·저크 반영).</t>
         </is>

</xml_diff>

<commit_message>
[cubicon] v1.5.1-rc7: support default off, raft layers 0
Adjust rc6: enable_support 1 -> 0 and raft_layers 3 -> 0 (support and raft off by default).
The other rc6 changes stay: support_on_build_plate_only 0, threshold 30, tree(auto),
raft_contact_distance 0.2, detect_overhang_wall 1.

Bump product version rc6 -> rc7; update Excel release notes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
+++ b/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1.5.1-rc6</t>
+          <t>1.5.1-rc7</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -547,7 +547,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -557,19 +557,19 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>서포트·라프트·오버행 기본값 변경 (기본 프로세스, 전 재료 공통)</t>
+          <t>서포트 기본 off · 라프트 레이어 0 으로 조정</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>cubicon common @base: 서포트 사용 off→on, 빌드플레이트에만 on→off, 임계각 15→30, 유형 normal(auto)→tree(auto), 라프트 접점 Z 0.1→0.2, 라프트 레이어 0→3, 오버행 벽 감지 off→on.</t>
+          <t>cubicon common @base: enable_support 1→0, raft_layers 3→0. rc6 의 서포트/라프트 나머지 변경(빌드플레이트 off, 임계각 30, tree(auto), 접점 0.2, 오버행 벽 감지 on)은 유지.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc6</t>
+          <t>1.5.1-rc7</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -589,19 +589,19 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc5 → rc6</t>
+          <t>제품 버전 rc6 → rc7</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>서포트 옵션 변경 반영.</t>
+          <t>서포트/라프트 기본값 조정.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>1.5.1-rc5</t>
+          <t>1.5.1-rc6</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -611,29 +611,29 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Process profile</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>빌드 시 patch 0008 충돌(U src/libslic3r/utils.cpp) 수정</t>
+          <t>서포트·라프트·오버행 기본값 변경 (기본 프로세스, 전 재료 공통)</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>build_win.ps1 이 소스를 인덱스로 리셋('git checkout -- src')해, git apply --3way 가 staged 로 남긴 옛 패치본이 새 패치와 충돌하던 문제. 'git checkout HEAD -- ...'(인덱스+워크트리 모두 HEAD로 리셋)로 변경해 매 빌드 pristine 보장.</t>
+          <t>cubicon common @base: 서포트 사용 off→on, 빌드플레이트에만 on→off, 임계각 15→30, 유형 normal(auto)→tree(auto), 라프트 접점 Z 0.1→0.2, 라프트 레이어 0→3, 오버행 벽 감지 off→on.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc5</t>
+          <t>1.5.1-rc6</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -653,19 +653,19 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc4 → rc5</t>
+          <t>제품 버전 rc5 → rc6</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>빌드 스크립트 패치충돌 수정 반영.</t>
+          <t>서포트 옵션 변경 반영.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>1.5.1-rc4</t>
+          <t>1.5.1-rc5</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -675,29 +675,29 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Process profile</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>정밀도(공차) 보정 기본 프로세스 반영 (전 재료 공통)</t>
+          <t>빌드 시 patch 0008 충돌(U src/libslic3r/utils.cpp) 수정</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>cubicon common @base: 코끼리발 보정 0.15→0.2 · 보정 레이어 2 · X-Y 구멍 보정 0.2 · X-Y 윤곽 보상 0.02 추가. resolution 0.012 · slice_closing 0.049 · EF density 100% · 정밀한 벽/정확한 Z · 원호맞춤 off 는 기존 일치. Rainbow PLA HS 공차 캘리브레이션 결과이며 공정 설정이라 전 재료에 공통 적용됨.</t>
+          <t>build_win.ps1 이 소스를 인덱스로 리셋('git checkout -- src')해, git apply --3way 가 staged 로 남긴 옛 패치본이 새 패치와 충돌하던 문제. 'git checkout HEAD -- ...'(인덱스+워크트리 모두 HEAD로 리셋)로 변경해 매 빌드 pristine 보장.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc4</t>
+          <t>1.5.1-rc5</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -717,19 +717,19 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc3 → rc4</t>
+          <t>제품 버전 rc4 → rc5</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>정밀도 공차 프로세스 반영.</t>
+          <t>빌드 스크립트 패치충돌 수정 반영.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>1.5.1-rc3</t>
+          <t>1.5.1-rc4</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -744,24 +744,24 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Filament profile</t>
+          <t>Process profile</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Rainbow PLA HS 캘리브레이션 확정값 반영</t>
+          <t>정밀도(공차) 보정 기본 프로세스 반영 (전 재료 공통)</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Cubicon Rainbow PLA HS @base: 최대 체적 속도 28→17 mm³/s(실측), Pressure Advance 0.03 신규 활성화. 온도(215/220)·베드(60)·유량비율(0.98)·후퇴(2mm 상속)는 캘리브레이션으로 적정 확인. 여전히 test-only. 상세: Rainbow PLA HS_ProfileUpdate_20260731_R0.pptx.</t>
+          <t>cubicon common @base: 코끼리발 보정 0.15→0.2 · 보정 레이어 2 · X-Y 구멍 보정 0.2 · X-Y 윤곽 보상 0.02 추가. resolution 0.012 · slice_closing 0.049 · EF density 100% · 정밀한 벽/정확한 Z · 원호맞춤 off 는 기존 일치. Rainbow PLA HS 공차 캘리브레이션 결과이며 공정 설정이라 전 재료에 공통 적용됨.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc3</t>
+          <t>1.5.1-rc4</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -781,76 +781,76 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc2 → rc3</t>
+          <t>제품 버전 rc3 → rc4</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Rainbow PLA HS 프로파일 캘리브레이션 반영.</t>
+          <t>정밀도 공차 프로세스 반영.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>1.5.1-rc2</t>
+          <t>1.5.1-rc3</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>G-code load</t>
+          <t>Filament profile</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>OrcaForCubicon(1.4.1 등) 및 신규 1.5.0 gcode 로드 실패 수정 (patch 0008 회귀 대응)</t>
+          <t>Rainbow PLA HS 캘리브레이션 확정값 반영</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>patch 0008 로 헤더를 '; generated by OrcaSlicer'로 바꾼 뒤, Config.cpp 의 로드 검증이 여전히 '; generated by OrcaForCubicon' 만 허용해 자기 파일조차 'Not a gcode file generated by OrcaForCubicon' 로 거부되던 문제. 검증에 '; generated by ' + SLIC3R_OFFICIAL_NAME('OrcaSlicer') 허용을 추가(patch 0008 갱신).</t>
+          <t>Cubicon Rainbow PLA HS @base: 최대 체적 속도 28→17 mm³/s(실측), Pressure Advance 0.03 신규 활성화. 온도(215/220)·베드(60)·유량비율(0.98)·후퇴(2mm 상속)는 캘리브레이션으로 적정 확인. 여전히 test-only. 상세: Rainbow PLA HS_ProfileUpdate_20260731_R0.pptx.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc2</t>
+          <t>1.5.1-rc3</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Installer / Runtime</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>WebView2 Evergreen 런타임 조건부 설치 추가 (마법사 blank 방지)</t>
+          <t>제품 버전 rc2 → rc3</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>WebView2Loader.dll 만으로는 부족 — 클린 PC에 WebView2 런타임이 없으면 설정 마법사가 blank. NSIS 에서 레지스트리(EdgeUpdate pv) 확인 후 미설치 시 MicrosoftEdgeWebview2Setup.exe 를 silent 설치. package_win.ps1 이 부트스트래퍼를 자동 다운로드해 번들. (VC++ CRT/.NET-런타임 이슈는 CopyRuntime+vc_redist 로 기존에 이미 처리됨)</t>
+          <t>Rainbow PLA HS 프로파일 캘리브레이션 반영.</t>
         </is>
       </c>
     </row>
@@ -867,29 +867,29 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>G-code load</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>제품 버전 rc1 → rc2</t>
+          <t>OrcaForCubicon(1.4.1 등) 및 신규 1.5.0 gcode 로드 실패 수정 (patch 0008 회귀 대응)</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>gcode 로드 수정 + WebView2 런타임 준비 반영.</t>
+          <t>patch 0008 로 헤더를 '; generated by OrcaSlicer'로 바꾼 뒤, Config.cpp 의 로드 검증이 여전히 '; generated by OrcaForCubicon' 만 허용해 자기 파일조차 'Not a gcode file generated by OrcaForCubicon' 로 거부되던 문제. 검증에 '; generated by ' + SLIC3R_OFFICIAL_NAME('OrcaSlicer') 허용을 추가(patch 0008 갱신).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>1.5.1-rc1</t>
+          <t>1.5.1-rc2</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -899,29 +899,29 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>version / release</t>
+          <t>Installer / Runtime</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>기본 버전 1.5.0 → 1.5.1 (다음 개발 사이클 시작)</t>
+          <t>WebView2 Evergreen 런타임 조건부 설치 추가 (마법사 blank 방지)</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>GitHub v1.5.0 발행 후 v1.5.1 을 추가 발행하여, v1.5.0 실행 시 업데이트 알림 팝업이 정상 동작하는지 end-to-end 검증하기 위한 버전 업. release 빌드 시 '1.5.1' 로 태깅.</t>
+          <t>WebView2Loader.dll 만으로는 부족 — 클린 PC에 WebView2 런타임이 없으면 설정 마법사가 blank. NSIS 에서 레지스트리(EdgeUpdate pv) 확인 후 미설치 시 MicrosoftEdgeWebview2Setup.exe 를 silent 설치. package_win.ps1 이 부트스트래퍼를 자동 다운로드해 번들. (VC++ CRT/.NET-런타임 이슈는 CopyRuntime+vc_redist 로 기존에 이미 처리됨)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc5</t>
+          <t>1.5.1-rc2</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -931,29 +931,29 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Splash</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>다크모드 스플래시 로고에서 legacy 'style' 문구 제거</t>
+          <t>제품 버전 rc1 → rc2</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>splash_logo_dark.png 가 큐비콘 legacy 'style CUBICON' 로고였음(Style 시리즈는 OrcaForCubicon 미지원). light 로고 기반으로 흰색 CUBICON 텍스트 + 컬러 아이콘의 다크모드 전용 로고로 교체(2495→2125px).</t>
+          <t>gcode 로드 수정 + WebView2 런타임 준비 반영.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc5</t>
+          <t>1.5.1-rc1</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -968,24 +968,24 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>version / release</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc4 → rc5</t>
+          <t>기본 버전 1.5.0 → 1.5.1 (다음 개발 사이클 시작)</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>다크모드 스플래시 로고 수정 반영.</t>
+          <t>GitHub v1.5.0 발행 후 v1.5.1 을 추가 발행하여, v1.5.0 실행 시 업데이트 알림 팝업이 정상 동작하는지 end-to-end 검증하기 위한 버전 업. release 빌드 시 '1.5.1' 로 태깅.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc4</t>
+          <t>1.5.0-rc5</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -995,29 +995,29 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Build / Filament</t>
+          <t>Splash</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>테스트 전용 필라멘트 분리 (test 빌드=포함 / release 빌드=제외)</t>
+          <t>다크모드 스플래시 로고에서 legacy 'style' 문구 제거</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>cubicon/version/test_only_filaments.txt 매니페스트에 나열한 미검증 필라멘트를 release 빌드에서만 제거(cubicon/scripts/prune_test_filaments.ps1, build_win.ps1 -BuildType release 에서 호출). SSOT(cubicon/resources)는 전부 유지 → test 빌드는 모두 포함. 현재 test 전용: Cubicon Rainbow PLA HS, Cubicon TPU-HS(+fdm_filament_tpu). 검증 완료 시 매니페스트에서 해당 줄만 삭제하면 정식 승격.</t>
+          <t>splash_logo_dark.png 가 큐비콘 legacy 'style CUBICON' 로고였음(Style 시리즈는 OrcaForCubicon 미지원). light 로고 기반으로 흰색 CUBICON 텍스트 + 컬러 아이콘의 다크모드 전용 로고로 교체(2495→2125px).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc4</t>
+          <t>1.5.0-rc5</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -1037,19 +1037,19 @@
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc3 → rc4</t>
+          <t>제품 버전 rc4 → rc5</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>테스트/정식 필라멘트 분리 기능 반영.</t>
+          <t>다크모드 스플래시 로고 수정 반영.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc3</t>
+          <t>1.5.0-rc4</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -1064,24 +1064,24 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Update check</t>
+          <t>Build / Filament</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>OrcaForCubicon 전용 업데이트 알림 기능 (OrcaSlicer 기본 체크 비활성화)</t>
+          <t>테스트 전용 필라멘트 분리 (test 빌드=포함 / release 빌드=제외)</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>실행 시 GitHub 최신 릴리스(api.github.com/repos/Hyvision/OrcaForCubicon/releases/latest)를 조회해 제품버전 CUBI_ORCA_VERSION 과 비교, 새 정식 릴리스가 있으면 팝업 알림 → '다운로드' 시 브라우저로 릴리스 페이지 열기. 정식 릴리스만 대상(/releases/latest 가 draft·prerelease 자동 제외). OrcaSlicer 의 check_new_version_sf 는 시작·수동 '업데이트 확인' 메뉴 양쪽에서 check_new_version_cubicon 으로 대체. 기존 UpdateVersionDialog 재사용. (patch 0009) ※ 동작하려면 레포 public 전환 + GitHub Releases 발행 필요.</t>
+          <t>cubicon/version/test_only_filaments.txt 매니페스트에 나열한 미검증 필라멘트를 release 빌드에서만 제거(cubicon/scripts/prune_test_filaments.ps1, build_win.ps1 -BuildType release 에서 호출). SSOT(cubicon/resources)는 전부 유지 → test 빌드는 모두 포함. 현재 test 전용: Cubicon Rainbow PLA HS, Cubicon TPU-HS(+fdm_filament_tpu). 검증 완료 시 매니페스트에서 해당 줄만 삭제하면 정식 승격.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc3</t>
+          <t>1.5.0-rc4</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1101,19 +1101,19 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc2 → rc3</t>
+          <t>제품 버전 rc3 → rc4</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>업데이트 알림 기능 추가 반영.</t>
+          <t>테스트/정식 필라멘트 분리 기능 반영.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc2</t>
+          <t>1.5.0-rc3</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -1123,29 +1123,29 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Feat</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>G-code / Mainsail</t>
+          <t>Update check</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>G-code 헤더 슬라이서명·버전 정정 (Moonraker 메타데이터 파싱 복원)</t>
+          <t>OrcaForCubicon 전용 업데이트 알림 기능 (OrcaSlicer 기본 체크 비활성화)</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>header_slic3r_generated() 가 "OrcaForCubicon 2.4.2" → "OrcaSlicer &lt;제품버전&gt;" 로 변경. Moonraker/Mainsail 은 인식된 슬라이서명(OrcaSlicer 등)일 때만 슬라이싱 정보를 파싱함 → 기존엔 Unknown+정보 없음. 버전도 Orca 2.4.2 대신 재정의 제품버전 표기. Orca 자체 재파싱은 GCodeProcessor 의 "generated by OrcaSlicer" producer 태그로 유지. (patch 0008)</t>
+          <t>실행 시 GitHub 최신 릴리스(api.github.com/repos/Hyvision/OrcaForCubicon/releases/latest)를 조회해 제품버전 CUBI_ORCA_VERSION 과 비교, 새 정식 릴리스가 있으면 팝업 알림 → '다운로드' 시 브라우저로 릴리스 페이지 열기. 정식 릴리스만 대상(/releases/latest 가 draft·prerelease 자동 제외). OrcaSlicer 의 check_new_version_sf 는 시작·수동 '업데이트 확인' 메뉴 양쪽에서 check_new_version_cubicon 으로 대체. 기존 UpdateVersionDialog 재사용. (patch 0009) ※ 동작하려면 레포 public 전환 + GitHub Releases 발행 필요.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc2</t>
+          <t>1.5.0-rc3</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1155,22 +1155,22 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>build_win.ps1</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>release / test 빌드 유형 옵션 추가</t>
+          <t>제품 버전 rc2 → rc3</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>-BuildType test|release (대화식 프롬프트 4번). release 는 버전의 -rc 접미사를 제거하여 splash·버전정보·About 대화상자·G-code 헤더·인스톨러명 모두에 반영. test 는 rc 유지. cubicon_version.txt(SSOT)를 빌드 중 임시 수정 후 finally 에서 원복.</t>
+          <t>업데이트 알림 기능 추가 반영.</t>
         </is>
       </c>
     </row>
@@ -1187,22 +1187,22 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>build_win.ps1</t>
+          <t>G-code / Mainsail</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>병렬 컴파일 잡을 메모리 기준으로도 제한 (-MemPerJobGB)</t>
+          <t>G-code 헤더 슬라이서명·버전 정정 (Moonraker 메타데이터 파싱 복원)</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>28코어/32GB 환경에서 CpuPercent 70%(=19잡)로 libslic3r PCH 컴파일 시 페이지파일 고갈(C3859/C1076/OS 1455) 발생. jobs = min(CPU 상한, floor((총RAM-4)/MemPerJobGB[기본3])) 로 제한하여 재발 방지.</t>
+          <t>header_slic3r_generated() 가 "OrcaForCubicon 2.4.2" → "OrcaSlicer &lt;제품버전&gt;" 로 변경. Moonraker/Mainsail 은 인식된 슬라이서명(OrcaSlicer 등)일 때만 슬라이싱 정보를 파싱함 → 기존엔 Unknown+정보 없음. 버전도 Orca 2.4.2 대신 재정의 제품버전 표기. Orca 자체 재파싱은 GCodeProcessor 의 "generated by OrcaSlicer" producer 태그로 유지. (patch 0008)</t>
         </is>
       </c>
     </row>
@@ -1219,29 +1219,29 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Chore</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>build_win.ps1</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>제품 버전 rc1 → rc2</t>
+          <t>release / test 빌드 유형 옵션 추가</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>cubicon/version/cubicon_version.txt. 규칙: 매 수정마다 rc 1 증가(반영 여부 식별용).</t>
+          <t>-BuildType test|release (대화식 프롬프트 4번). release 는 버전의 -rc 접미사를 제거하여 splash·버전정보·About 대화상자·G-code 헤더·인스톨러명 모두에 반영. test 는 rc 유지. cubicon_version.txt(SSOT)를 빌드 중 임시 수정 후 finally 에서 원복.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>1.5.0-rc1</t>
+          <t>1.5.0-rc2</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -1251,29 +1251,29 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Machine profile</t>
+          <t>build_win.ps1</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>장비 Max Jerk 하향 (Bambu·Creality 기조: 고가감속·저저크)</t>
+          <t>병렬 컴파일 잡을 메모리 기준으로도 제한 (-MemPerJobGB)</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>xCeler-Plus/I/Mini 3종: X 20→5, Y 20→5, Z 20→2, E 20→2.5 mm/s. 캔틸레버 베드 편심 틸트로 레이어 중 Z가 상시 반전할 때 높은 Z 저크가 임펄스 진동→수직 벽면 잔상(ghosting)을 유발하던 문제 해결. 장비 프로파일 version → 1.5.0.</t>
+          <t>28코어/32GB 환경에서 CpuPercent 70%(=19잡)로 libslic3r PCH 컴파일 시 페이지파일 고갈(C3859/C1076/OS 1455) 발생. jobs = min(CPU 상한, floor((총RAM-4)/MemPerJobGB[기본3])) 로 제한하여 재발 방지.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>1.5.0-rc1</t>
+          <t>1.5.0-rc2</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
@@ -1283,22 +1283,22 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Feat</t>
+          <t>Chore</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Filament profile</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>신규 필라멘트: Cubicon TPU-HS</t>
+          <t>제품 버전 rc1 → rc2</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>isun3d TPU-HS(고속 TPU, Shore 95A) 추가. base + xCeler-I/Plus/Mini. fdm_filament_tpu 계열 베이스 신설. 초기값(노즐 230/230, 베드 50, 최대유량 5, 팬 100%) — 캘리브레이션 예정.</t>
+          <t>cubicon/version/cubicon_version.txt. 규칙: 매 수정마다 rc 1 증가(반영 여부 식별용).</t>
         </is>
       </c>
     </row>
@@ -1320,17 +1320,17 @@
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Filament profile</t>
+          <t>Machine profile</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>신규 필라멘트: Cubicon Rainbow PLA HS</t>
+          <t>장비 Max Jerk 하향 (Bambu·Creality 기조: 고가감속·저저크)</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>한일 Rainbow PLA High Speed (Bambu PLA HS 유사). base + xCeler-I/Plus/Mini, Cubicon PLA @base 상속. 초기값(노즐 220/215, 베드 60, 최대유량 28, flow 0.98) — 캘리브레이션 예정.</t>
+          <t>xCeler-Plus/I/Mini 3종: X 20→5, Y 20→5, Z 20→2, E 20→2.5 mm/s. 캔틸레버 베드 편심 틸트로 레이어 중 Z가 상시 반전할 때 높은 Z 저크가 임펄스 진동→수직 벽면 잔상(ghosting)을 유발하던 문제 해결. 장비 프로파일 version → 1.5.0.</t>
         </is>
       </c>
     </row>
@@ -1347,20 +1347,84 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
+          <t>Feat</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Filament profile</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>신규 필라멘트: Cubicon TPU-HS</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>isun3d TPU-HS(고속 TPU, Shore 95A) 추가. base + xCeler-I/Plus/Mini. fdm_filament_tpu 계열 베이스 신설. 초기값(노즐 230/230, 베드 50, 최대유량 5, 팬 100%) — 캘리브레이션 예정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>1.5.0-rc1</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Feat</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Filament profile</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>신규 필라멘트: Cubicon Rainbow PLA HS</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>한일 Rainbow PLA High Speed (Bambu PLA HS 유사). base + xCeler-I/Plus/Mini, Cubicon PLA @base 상속. 초기값(노즐 220/215, 베드 60, 최대유량 28, flow 0.98) — 캘리브레이션 예정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>1.5.0-rc1</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
           <t>Chore</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="D32" s="7" t="inlineStr">
         <is>
           <t>Profile package</t>
         </is>
       </c>
-      <c r="E30" s="7" t="inlineStr">
+      <c r="E32" s="7" t="inlineStr">
         <is>
           <t>프로파일 패키지 버전 02.03.02.00 → 02.03.03.00</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
+      <c r="F32" s="7" t="inlineStr">
         <is>
           <t>Cubicon.json. 기설치 사용자에게 프로파일 갱신 전파를 위해 패키지 버전 상승 (신규 필라멘트·저크 반영).</t>
         </is>

</xml_diff>

<commit_message>
[cubicon] docs: condense the customer-facing release-notes sheet
"Release Notes (Simple)" is handed to end customers, so it should read at a glance:
one or two lines per shipped version instead of a per-change table. Dropped the
Type / customer-impact columns (3 columns left: 버전 / 배포일 / 주요 변경 사항) and
folded the 1.5.1 items into two lines, 1.5.0 into two.

"Release Notes (Detail)" (full per-rc log) and "Jerk Parameters" are unchanged.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
+++ b/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
@@ -104,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -138,6 +138,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -504,14 +510,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="66" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="84" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -524,7 +528,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>최신 버전 1.5.1 (2026-08-11) · OrcaSlicer 2.4.2 기반 · 대상 장비: Cubicon xCeler-Plus / xCeler-I / xCeler-Mini</t>
+          <t>최신 버전 1.5.1 (2026-08-11) · 대상 장비: Cubicon xCeler-Plus / xCeler-I / xCeler-Mini</t>
         </is>
       </c>
     </row>
@@ -541,17 +545,7 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>구분</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
           <t>주요 변경 사항</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>고객 영향 / 설명</t>
         </is>
       </c>
     </row>
@@ -566,19 +560,9 @@
           <t>2026-08-11</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>수정</t>
-        </is>
-      </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>G-code 파일 열기 호환성 복원</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>이전 버전(1.4.x)이나 OrcaSlicer 에서 저장한 G-code 를 다시 불러올 수 있습니다. 1.5.0 에서 "OrcaForCubicon 에서 생성한 gcode 파일이 아닙니다" 오류로 열리지 않던 문제를 수정했습니다.</t>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>이전 버전(1.4.x)·OrcaSlicer 에서 저장한 G-code 파일이 열리지 않던 문제 수정, 새 PC 설치 안정화</t>
         </is>
       </c>
     </row>
@@ -593,247 +577,48 @@
           <t>2026-08-11</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>수정</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Mainsail / Moonraker 슬라이싱 정보 표시</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="inlineStr">
-        <is>
-          <t>프린터 웹 UI 에서 슬라이서 이름·버전과 출력 정보가 정상적으로 표시됩니다.</t>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>출력 정밀도(공차) 보정 기본 적용 및 서포트·라프트 기본값 정리</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>1.5.1</t>
+          <t>1.5.0</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>설치</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="inlineStr">
-        <is>
-          <t>새 PC 설치 안정화 (WebView2 런타임 자동 설치)</t>
-        </is>
-      </c>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>설치 시 필요한 WebView2 런타임을 자동으로 함께 설치합니다. 새 PC 에서 최초 실행 시 설정 마법사가 빈 화면으로 표시되던 문제가 해결됩니다. (VC++ 런타임도 동봉)</t>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>출력 품질 개선 — Z축 벽면 잔상(고스팅) 저감</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>1.5.1</t>
+          <t>1.5.0</t>
         </is>
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>개선</t>
-        </is>
-      </c>
-      <c r="D8" s="13" t="inlineStr">
-        <is>
-          <t>출력 정밀도(공차) 기본값 보정</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="inlineStr">
-        <is>
-          <t>코끼리발 보정 및 X-Y 구멍/외곽 보정을 기본 프로파일에 적용했습니다. 구멍 지름과 외곽 치수 정확도가 향상됩니다. (모든 재료 공통 적용)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>1.5.1</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>개선</t>
-        </is>
-      </c>
-      <c r="D9" s="11" t="inlineStr">
-        <is>
-          <t>서포트 · 라프트 · 오버행 기본값 정리</t>
-        </is>
-      </c>
-      <c r="E9" s="11" t="inlineStr">
-        <is>
-          <t>서포트 기본 끔, 라프트 0층으로 설정했습니다. 서포트를 켤 경우 유형은 트리(자동), 임계각 30° 가 기본이며 오버행 감지가 켜집니다.</t>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>새 버전 업데이트 알림 기능 추가</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>1.5.1</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="C10" s="12" t="inlineStr">
-        <is>
-          <t>개선</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>시작 화면(스플래시) 개선</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>CUBICON 과 Orca 로고를 함께 표시하고 제품명 "OrcaForCubicon" 을 표기합니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>1.5.0</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>개선</t>
-        </is>
-      </c>
-      <c r="D11" s="11" t="inlineStr">
-        <is>
-          <t>출력 품질 개선 — 장비 저크(Jerk) 하향 조정</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="inlineStr">
-        <is>
-          <t>Z축 벽면 잔상(고스팅)이 줄어듭니다. xCeler-Plus / I / Mini 공통 적용이며, G-code 에 자동 반영되므로 장비 설정을 따로 바꿀 필요가 없습니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>1.5.0</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>신규</t>
-        </is>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>업데이트 알림</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="inlineStr">
-        <is>
-          <t>새 버전이 배포되면 프로그램 시작 시 안내 팝업이 표시되고, 클릭하면 다운로드 페이지로 이동합니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>1.5.0</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>개선</t>
-        </is>
-      </c>
-      <c r="D13" s="11" t="inlineStr">
-        <is>
-          <t>큐비콘 프로파일 패키지 갱신 (02.03.03.00)</t>
-        </is>
-      </c>
-      <c r="E13" s="11" t="inlineStr">
-        <is>
-          <t>기존 설치 사용자에게도 갱신된 큐비콘 장비·재료 프로파일이 전파됩니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>1.5.0</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>수정</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="inlineStr">
-        <is>
-          <t>다크 모드 시작 화면 로고</t>
-        </is>
-      </c>
-      <c r="E14" s="13" t="inlineStr">
-        <is>
-          <t>다크 모드에서 구형 "style CUBICON" 로고가 표시되던 문제를 수정했습니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>※ 시험 중인 필라멘트(Rainbow PLA HS, TPU-HS)는 검증 완료 전까지 정식 배포판에 포함되지 않습니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>※ 다운로드: https://github.com/Hyvision/OrcaForCubicon/releases/latest</t>
         </is>

</xml_diff>

<commit_message>
[cubicon] stay on 1.5.2: version 1.5.3-rc1 -> 1.5.2-rc3
Keep the filament-visibility fix inside the 1.5.2 line instead of opening a 1.5.3
cycle. cubicon_version.txt goes to 1.5.2-rc3 and the release-notes rows added for
1.5.3-rc1 are relabelled 1.5.2-rc3 (Detail) / 1.5.2 (Simple). A release build strips
the rc suffix, so the app still reports 1.5.2.

The profile package stays at 02.03.05.00 -- 02.03.04.00 already shipped in the
published v1.5.2, so installed users still need the bump to pick up the corrected
machine models.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
+++ b/cubicon/doc/OrcaForCubicon_ReleaseNotes.xlsx
@@ -528,7 +528,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>최신 버전 1.5.3 (2026-08-20) · 대상 장비: Cubicon xCeler-Plus / xCeler-I / xCeler-Mini</t>
+          <t>최신 버전 1.5.2 · 대상 장비: Cubicon xCeler-Plus / xCeler-I / xCeler-Mini</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>1.5.3</t>
+          <t>1.5.2</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
@@ -732,7 +732,7 @@
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>1.5.3-rc1</t>
+          <t>1.5.2-rc3</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
@@ -764,7 +764,7 @@
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>1.5.3-rc1</t>
+          <t>1.5.2-rc3</t>
         </is>
       </c>
       <c r="B6" s="12" t="inlineStr">
@@ -796,7 +796,7 @@
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>1.5.3-rc1</t>
+          <t>1.5.2-rc3</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
@@ -816,12 +816,12 @@
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>기본 버전 1.5.2 → 1.5.3 (다음 개발 사이클 시작)</t>
+          <t>제품 버전 rc2 → rc3</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>v1.5.2 GitHub 릴리스 발행 완료에 따라 1.5.3-rc1 로 전환.</t>
+          <t>v1.5.2 발행 이후의 수정이지만 버전 번호는 1.5.2 를 유지하고 rc 만 상승. release 빌드가 rc 접미사를 제거하므로 앱 표시 버전은 1.5.2 그대로.</t>
         </is>
       </c>
     </row>

</xml_diff>